<commit_message>
feat: mostra a origem de cada entrada da planilha V3.0 (FB-02, FB-03, FB-06)
Feedback da equipe: não dava para distinguir dado firme de estimado nem
saber de onde veio cada valor, as cores confundiam e a orientação ficava
fora da planilha.

- Colunas Origem (lista "Origens" com 6 rótulos e símbolo) e Fonte em cada
  entrada de 05, 06, 07, 08 e 11, e I/J na 10_TIRE; os comentários viraram
  a Fonte. Cor só na Origem; aviso de origem desatualizada e de "Dado do TX"
  sem fonte por formatação condicional (G/H ocultas). EDR-035, EDR-025 = A.
- Fundo amarelo "hipótese-chave" retirado; legenda com o estilo real.
- Guia "Como preencher" na 00_README (inclui o aviso do EDR-051).
- TC-WB30-010 a 012. Nenhuma fórmula muda (356); suíte inteira PASS.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel/FSAE_EV_Suspension_Fase1_V3_0.xlsx
+++ b/excel/FSAE_EV_Suspension_Fase1_V3_0.xlsx
@@ -24,7 +24,9 @@
     <sheet name="14_DASHBOARD" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="15_CHANGELOG" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="Origens">'00_README'!$A$43:$A$48</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -173,7 +175,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -246,10 +248,70 @@
     <xf numFmtId="1" fontId="8" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="6">
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="00FFFFFF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00D55E00"/>
+          <bgColor rgb="00D55E00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00CCE3F0"/>
+          <bgColor rgb="00CCE3F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FAE2B3"/>
+          <bgColor rgb="00FAE2B3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00F0D7E5"/>
+          <bgColor rgb="00F0D7E5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00E0E0E0"/>
+          <bgColor rgb="00E0E0E0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FF0000"/>
+          <bgColor rgb="00FF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -349,66 +411,6 @@
     <author>Engineering Standard v0.1</author>
   </authors>
   <commentList>
-    <comment ref="B4" authorId="0" shapeId="0">
-      <text>
-        <t>Fonte: adesivo SAE Brasil 2026 - medicao real (248.5 kg sem piloto) + 68 kg de piloto (referencia padrao FSAE, nao medida).</t>
-      </text>
-    </comment>
-    <comment ref="B5" authorId="0" shapeId="0">
-      <text>
-        <t>Fonte: E05 (315mm, Key Parameters). Medida a partir do plano do solo (SUS-000), nao da origem do CAD.</t>
-      </text>
-    </comment>
-    <comment ref="B6" authorId="0" shapeId="0">
-      <text>
-        <t>Fonte: E05 (1594mm, Key Parameters). Diverge do E03 (1550mm, chassi anterior).</t>
-      </text>
-    </comment>
-    <comment ref="B7" authorId="0" shapeId="0">
-      <text>
-        <t>Fonte: E05 (1277mm, Key Parameters).</t>
-      </text>
-    </comment>
-    <comment ref="B8" authorId="0" shapeId="0">
-      <text>
-        <t>Fonte: E05 (1271mm, Key Parameters).</t>
-      </text>
-    </comment>
-    <comment ref="B9" authorId="0" shapeId="0">
-      <text>
-        <t>Derivado da distribuicao real medida no adesivo TX/E05 (48.43% dianteira, COM piloto) x wheelbase - consistente com mass_total (que inclui piloto).</t>
-      </text>
-    </comment>
-    <comment ref="B10" authorId="0" shapeId="0">
-      <text>
-        <t>Derivado da distribuicao real medida no adesivo TX/E05 (51.57% traseira, COM piloto) x wheelbase.</t>
-      </text>
-    </comment>
-    <comment ref="B14" authorId="0" shapeId="0">
-      <text>
-        <t>NAO DISPONIVEL para o TX/E05 (confirmado pela equipe: pesagem em plataforma mede carga total no solo, nao separa massa suspensa/nao-suspensa). Valor abaixo e ARBITRARIO - nao usar para decisao de projeto.</t>
-      </text>
-    </comment>
-    <comment ref="B15" authorId="0" shapeId="0">
-      <text>
-        <t>NAO DISPONIVEL para o TX/E05 (mesma razao do SUS-007). Valor abaixo e ARBITRARIO - nao usar para decisao de projeto.</t>
-      </text>
-    </comment>
-    <comment ref="B16" authorId="0" shapeId="0">
-      <text>
-        <t>Estimativa pelo raio do pneu 20.0-13 (E03, diametro 20.0in/2=0.254m). NAO e medicao real da equipe.</t>
-      </text>
-    </comment>
-    <comment ref="B17" authorId="0" shapeId="0">
-      <text>
-        <t>Estimativa pelo raio do pneu 20.0-13 (E03, mesmo pneu dianteiro/traseiro). NAO e medicao real da equipe.</t>
-      </text>
-    </comment>
-    <comment ref="B20" authorId="0" shapeId="0">
-      <text>
-        <t>SUS-000: coordenada Z do solo no sistema de coordenadas da equipe. Todas as alturas desta planilha já assumem conversão feita (medidas a partir do solo). Ver Engineering Standard, ficha SUS-000.</t>
-      </text>
-    </comment>
     <comment ref="B24" authorId="0" shapeId="0">
       <text>
         <t>h_s != h_CG total. Identidade de CG composto (verificada algebricamente na arquitetura, seção 17.4).</t>
@@ -421,83 +423,17 @@
 <file path=xl/comments/comment3.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
-    <author>Sistema_DDS V3.0</author>
     <author>Engineering Standard v0.1</author>
   </authors>
   <commentList>
-    <comment ref="B4" authorId="0" shapeId="0">
-      <text>
-        <t>DEMONSTRATIVO (EDR-012/022): valor herdado do T09/E03, usado só para referência, comparação e teste das fórmulas (confirmado pelo usuário em 2026-10-19). Não é o TX/E05. Back-calculado da planilha detalhada T09 ('Ride Rate' front=16112.23 N/m, confirmado ser exatamente o Wheel Rate) x MR=1.76. CORRIGE valor anterior (baseado no spec sheet resumido, que arredondava F/R como iguais).</t>
-      </text>
-    </comment>
-    <comment ref="B5" authorId="0" shapeId="0">
-      <text>
-        <t>DEMONSTRATIVO (EDR-012/022): valor herdado do T09/E03, usado só para referência, comparação e teste das fórmulas (confirmado pelo usuário em 2026-10-19). Não é o TX/E05. Back-calculado da planilha detalhada T09 ('Ride Rate' rear=18418.2 N/m) x MR=1.76.</t>
-      </text>
-    </comment>
-    <comment ref="B6" authorId="0" shapeId="0">
-      <text>
-        <t>DEMONSTRATIVO (EDR-012/022): valor herdado do T09/E03, usado só para referência, comparação e teste das fórmulas (confirmado pelo usuário em 2026-10-19). Não é o TX/E05. Fonte: E03 (1.76:1). Assumido como convencao wheel/spring (igual a nossa) - E03 nao especifica a direcao explicitamente.</t>
-      </text>
-    </comment>
-    <comment ref="B7" authorId="0" shapeId="0">
-      <text>
-        <t>DEMONSTRATIVO (EDR-012/022): valor herdado do T09/E03, usado só para referência, comparação e teste das fórmulas (confirmado pelo usuário em 2026-10-19). Não é o TX/E05. Fonte: E03 (1.76:1, mesmo valor da dianteira).</t>
-      </text>
-    </comment>
-    <comment ref="B10" authorId="0" shapeId="0">
-      <text>
-        <t>DEMONSTRATIVO (EDR-012/022): valor herdado do T09/E03, usado só para referência, comparação e teste das fórmulas (confirmado pelo usuário em 2026-10-19). Não é o TX/E05. Fonte: planilha detalhada T09 (AntiRoll Bar Rate front). Valor direto, ja nao e mais back-calculado - resolve a inconsistencia identificada anteriormente.</t>
-      </text>
-    </comment>
-    <comment ref="B11" authorId="0" shapeId="0">
-      <text>
-        <t>DEMONSTRATIVO (EDR-012/022): valor herdado do T09/E03, usado só para referência, comparação e teste das fórmulas (confirmado pelo usuário em 2026-10-19). Não é o TX/E05. Fonte: planilha detalhada T09 (AntiRoll Bar Rate rear, ~0, consistente com 'sem ARB' declarado). Inconsistencia anterior estava no Wheel Rate do spec sheet resumido, ja corrigida em SUS-203.</t>
-      </text>
-    </comment>
-    <comment ref="B14" authorId="0" shapeId="0">
-      <text>
-        <t>DEMONSTRATIVO (EDR-012/022): valor herdado do T09/E03, usado só para referência, comparação e teste das fórmulas (confirmado pelo usuário em 2026-10-19). Não é o TX/E05. Fonte: planilha detalhada T09 (0.0675m) - mais precisa que o spec sheet resumido do E03 (60mm, arredondado). PROVISORIO ate Fase 2 (OptimumKinematics).</t>
-      </text>
-    </comment>
-    <comment ref="B15" authorId="0" shapeId="0">
-      <text>
-        <t>DEMONSTRATIVO (EDR-012/022): valor herdado do T09/E03, usado só para referência, comparação e teste das fórmulas (confirmado pelo usuário em 2026-10-19). Não é o TX/E05. Fonte: E03 (110mm, Roll center height above ground static). PROVISORIO ate Fase 2 (OptimumKinematics).</t>
-      </text>
-    </comment>
-    <comment ref="B20" authorId="1" shapeId="0">
+    <comment ref="B20" authorId="0" shapeId="0">
       <text>
         <t>Componente so-mola, sem ARB. Mesma decomposicao ja verificada 7/7 no T09 Reference Case.</t>
       </text>
     </comment>
-    <comment ref="B36" authorId="1" shapeId="0">
-      <text>
-        <t>PLACEHOLDER: fracao da forca de frenagem no eixo dianteiro (brake bias). Substituir pelo balanco de freio real do Setup.</t>
-      </text>
-    </comment>
-    <comment ref="B37" authorId="1" shapeId="0">
-      <text>
-        <t>TF_r = 1 para RWD (hipotese congelada da V1). Revisitar se a equipe migrar para AWD.</t>
-      </text>
-    </comment>
-    <comment ref="B40" authorId="1" shapeId="0">
+    <comment ref="B40" authorId="0" shapeId="0">
       <text>
         <t>AD_f = FB_f * tan(phi_f) * (L/hCG) * 100. NAO altera a magnitude do load transfer longitudinal (SUS-102) - so descreve particao geometrica vs. elastica.</t>
-      </text>
-    </comment>
-    <comment ref="B44" authorId="1" shapeId="0">
-      <text>
-        <t>PLACEHOLDER: razao entre angulo do volante e angulo medio das rodas dianteiras. Substituir por medicao real da cremalheira ou geometria do rack.</t>
-      </text>
-    </comment>
-    <comment ref="B47" authorId="0" shapeId="0">
-      <text>
-        <t>PROVISÓRIO (EDR-045): VERTICAL_STIFFNESS do .tir TTC provisório (Hoosier R25B, EDR-038). Não é o pneu do carro nem medição da equipe: substituir pela rigidez vertical do pneu real. Milliken p. 591, Gillespie eq. 5-8 e Seward eq. 4.1 põem o pneu em série com a mola.</t>
-      </text>
-    </comment>
-    <comment ref="B48" authorId="0" shapeId="0">
-      <text>
-        <t>PROVISÓRIO (EDR-045): VERTICAL_STIFFNESS do .tir TTC provisório (Hoosier R25B, EDR-038). Não é o pneu do carro nem medição da equipe: substituir pela rigidez vertical do pneu real. Milliken p. 591, Gillespie eq. 5-8 e Seward eq. 4.1 põem o pneu em série com a mola.</t>
       </text>
     </comment>
   </commentList>
@@ -508,7 +444,6 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Engineering Standard v0.1</author>
-    <author>Sistema_DDS V3.0</author>
   </authors>
   <commentList>
     <comment ref="B7" authorId="0" shapeId="0">
@@ -516,46 +451,11 @@
         <t>V1 usa apenas o KOP de ride height estatico. Curvas ao longo do curso (bump/rebound) ficam para Fase 2.</t>
       </text>
     </comment>
-    <comment ref="B10" authorId="0" shapeId="0">
-      <text>
-        <t>PLACEHOLDER geometrico para teste de formula - NAO e hardpoint real. Fase 2: REFERENCE do OptimumKinematics.</t>
-      </text>
-    </comment>
-    <comment ref="B14" authorId="1" shapeId="0">
-      <text>
-        <t>PLACEHOLDER: usa a altura do CG não suspenso traseiro (SUS-011), que a ficha aproxima pela altura do centro da roda. Substituir pela altura do centro da roda do CAD.</t>
-      </text>
-    </comment>
-    <comment ref="B31" authorId="0" shapeId="0">
-      <text>
-        <t>PLACEHOLDER geometrico - NAO e medicao real do curso instalado. Substituir pelo curso real (bump+rebound) com piloto sentado, conforme V.3.1.1.</t>
-      </text>
-    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/comments/comment5.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Engineering Standard v0.1</author>
-  </authors>
-  <commentList>
-    <comment ref="B4" authorId="0" shapeId="0">
-      <text>
-        <t>ISO 8855: a_x positivo = aceleração para frente (transfere carga para o eixo traseiro). Negativo = frenagem.</t>
-      </text>
-    </comment>
-    <comment ref="B5" authorId="0" shapeId="0">
-      <text>
-        <t>ISO 8855: a_y positivo = para a esquerda (lado direito do carro ganha carga).</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment6.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Sistema_DDS V2.2</author>
@@ -591,26 +491,11 @@
         <t>Coluna VERIF: caso fixo (Fz=700 N, α=3°, γ=1,5°, κ=0,05, roda direita) cujo resultado é comparado ao de tire_model_V2_2.py em 13_VALIDATION. Não representa o carro.</t>
       </text>
     </comment>
-    <comment ref="B23" authorId="0" shapeId="0">
-      <text>
-        <t>DEMONSTRATIVOS (EDR-022): α, γ e κ não vêm de nenhum cálculo do carro (não há modelo de slip na V2). Valores arbitrários coerentes em sinal com 08_VEHICLE_STATE (curva à esquerda, frenagem). Substitua por casos de carga definidos pela equipe.</t>
-      </text>
-    </comment>
-    <comment ref="B24" authorId="0" shapeId="0">
-      <text>
-        <t>Camber de entrada manual (EDR-036 sem decisão: ainda não há ID para camber estático). Convenção do projeto: + = topo para fora, nos dois lados.</t>
-      </text>
-    </comment>
-    <comment ref="B86" authorId="0" shapeId="0">
-      <text>
-        <t>Todos os coeficientes desta tabela: transcritos do .tir provisório (ver B-metadados). REFERENCE por natureza (DR-011), mas o DATASET é PROVISÓRIO. Mudou o dataset =&gt; mudar Tire REV (01_SETUP) e reexecutar 13_VALIDATION; resultados antigos viram STALE (Guia, H.3).</t>
-      </text>
-    </comment>
   </commentList>
 </comments>
 </file>
 
-<file path=xl/comments/comment7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments/comment6.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Engineering Standard v0.1</author>
@@ -625,7 +510,7 @@
 </comments>
 </file>
 
-<file path=xl/comments/comment8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments/comment7.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Engineering Standard v0.1</author>
@@ -940,7 +825,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -957,13 +842,15 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Versão do workbook: V3.0 (em desenvolvimento até concluir as correções de feedback; revisão metodológica contra Milliken/Gillespie/Seward/Pacejka: pneu em série, termo gravitacional da rolagem, massa suspensa por eixo, anti com sinal, Ky com um λFz0; EDR-045 a EDR-049) | Status: DRAFT — cross-check, ainda NÃO REFERENCE-validated</t>
-        </is>
-      </c>
-    </row>
+          <t>Versão do workbook: V3.0 (em desenvolvimento até concluir as correções de feedback; revisão metodológica contra Milliken/Gillespie/Seward/Pacejka: pneu em série, termo gravitacional da rolagem, massa suspensa por eixo, anti com sinal, Ky com um λFz0; EDR-045 a EDR-049; 2ª rodada, feedback da equipe: origem de cada entrada, guia de preenchimento; EDR-035, EDR-051) | Status: DRAFT — cross-check, ainda NÃO REFERENCE-validated</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
@@ -1023,6 +910,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
@@ -1031,7 +919,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="inlineStr">
+      <c r="A16" s="16" t="inlineStr">
         <is>
           <t>■ Azul</t>
         </is>
@@ -1043,7 +931,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="inlineStr">
+      <c r="A17" s="17" t="inlineStr">
         <is>
           <t>■ Verde-teal</t>
         </is>
@@ -1055,7 +943,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="inlineStr">
+      <c r="A18" s="22" t="inlineStr">
         <is>
           <t>■ Laranja + fundo</t>
         </is>
@@ -1067,7 +955,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="inlineStr">
+      <c r="A19" s="21" t="inlineStr">
         <is>
           <t>■ Preto + fundo cinza</t>
         </is>
@@ -1079,17 +967,18 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>■ Amarelo</t>
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Origem do valor</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Hipótese-chave / célula de atenção</t>
-        </is>
-      </c>
-    </row>
+          <t>Não é cor da célula: fica na coluna E de cada entrada (● ◐ ○ ?). Ver "Como preencher", abaixo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
@@ -1139,6 +1028,7 @@
         </is>
       </c>
     </row>
+    <row r="29"/>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
@@ -1195,39 +1085,216 @@
         </is>
       </c>
     </row>
+    <row r="38"/>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>Como preencher esta planilha (EDR-035, EDR-051)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>1. Edite só as entradas (fonte azul; verde-teal e laranja quando houver o dado real) das abas 05, 06, 07, 08, 10 (casos de carga) e 11 (metas). Célula com fundo cinza é calculada: não edite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>2. Cada entrada tem ao lado a Origem (coluna E; na 10_TIRE, coluna I) e a Fonte (coluna F; na 10_TIRE, J). Ao trocar um valor, escolha a Origem na lista e escreva na Fonte de onde veio o número. Origens possíveis:</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="30" customHeight="1">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Origem</t>
+        </is>
+      </c>
+      <c r="B42" s="44" t="inlineStr">
+        <is>
+          <t>Significado</t>
+        </is>
+      </c>
+      <c r="E42" s="44" t="inlineStr">
+        <is>
+          <t>Categorias da auditoria V2.1 (data/placeholder-dependency-map-V2.1.csv)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="30" customHeight="1">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>● Dado do TX</t>
+        </is>
+      </c>
+      <c r="B43" s="44" t="inlineStr">
+        <is>
+          <t>Medido no carro atual ou tirado de documento do TX/E05 (ex.: Key Parameters).</t>
+        </is>
+      </c>
+      <c r="E43" s="44" t="inlineStr">
+        <is>
+          <t>T3_FONTE_TX_REGISTRADA (T3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="30" customHeight="1">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>◐ Dado do T09</t>
+        </is>
+      </c>
+      <c r="B44" s="44" t="inlineStr">
+        <is>
+          <t>Valor do carro anterior (T09/E03): serve para testar as fórmulas, não é o TX.</t>
+        </is>
+      </c>
+      <c r="E44" s="44" t="inlineStr">
+        <is>
+          <t>REAL_OUTRO_VEICULO_T09/E03 (T2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="30" customHeight="1">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>◐ Provisório (.tir TTC)</t>
+        </is>
+      </c>
+      <c r="B45" s="44" t="inlineStr">
+        <is>
+          <t>Vem do arquivo de pneu provisório do TTC; não é o pneu do carro.</t>
+        </is>
+      </c>
+      <c r="E45" s="44" t="inlineStr">
+        <is>
+          <t>REAL_OUTRO_VEICULO_PROVISORIO (T2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="30" customHeight="1">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>○ Estimativa</t>
+        </is>
+      </c>
+      <c r="B46" s="44" t="inlineStr">
+        <is>
+          <t>Estimado ou suposto: inclui hipótese de modelo e caso de carga sem fonte.</t>
+        </is>
+      </c>
+      <c r="E46" s="44" t="inlineStr">
+        <is>
+          <t>ESTIMATIVA_NAO_MEDIDA (T1), HIPOTESE_CONGELADA_V1 e CASO_DE_CARGA_SEM_PROVENIENCIA (T2); vale a pior, T1</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="30" customHeight="1">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
+      <c r="B47" s="44" t="inlineStr">
+        <is>
+          <t>Placeholder, valor arbitrário ou meta de exemplo: não usar para decisão de projeto.</t>
+        </is>
+      </c>
+      <c r="E47" s="44" t="inlineStr">
+        <is>
+          <t>ARBITRARIO, PLACEHOLDER, ALVO_DEMONSTRATIVO (T1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="30" customHeight="1">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>? A confirmar</t>
+        </is>
+      </c>
+      <c r="B48" s="44" t="inlineStr">
+        <is>
+          <t>A origem do valor não está registrada.</t>
+        </is>
+      </c>
+      <c r="E48" s="44" t="inlineStr">
+        <is>
+          <t>sem classificação</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>3. Avisos: Origem com fundo vermelho-alaranjado = o valor mudou e a Origem continuou a mesma (revise a Origem). Fonte com fundo vermelho = a Origem diz "Dado do TX" e falta a Fonte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>4. Até a V3.0 ser fechada, esta planilha é gerada pelo script do repositório e o que for digitado nela se perde na próxima geração (EDR-051). Depois do fechamento, ela passa a ser o arquivo da equipe.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>5. Convenções de sinais e eixos: seção acima. Decisões e fichas: pasta docs/ do repositório (Engineering_Decision_Register.md e Engineering Standard).</t>
+        </is>
+      </c>
+    </row>
+    <row r="52"/>
   </sheetData>
-  <mergeCells count="31">
+  <mergeCells count="45">
     <mergeCell ref="A30:E30"/>
+    <mergeCell ref="A39:E39"/>
     <mergeCell ref="A34:E34"/>
+    <mergeCell ref="B42:D42"/>
     <mergeCell ref="A24:E24"/>
     <mergeCell ref="A15:E15"/>
     <mergeCell ref="A11:E11"/>
+    <mergeCell ref="A49:E49"/>
+    <mergeCell ref="A51:E51"/>
     <mergeCell ref="A1:E1"/>
+    <mergeCell ref="B44:D44"/>
     <mergeCell ref="A36:E36"/>
     <mergeCell ref="B20:E20"/>
     <mergeCell ref="A6:E6"/>
     <mergeCell ref="A7:E7"/>
     <mergeCell ref="A25:E25"/>
+    <mergeCell ref="A41:E41"/>
     <mergeCell ref="B16:E16"/>
     <mergeCell ref="A37:E37"/>
     <mergeCell ref="A27:E27"/>
     <mergeCell ref="A12:E12"/>
     <mergeCell ref="B18:E18"/>
+    <mergeCell ref="A50:E50"/>
     <mergeCell ref="A26:E26"/>
+    <mergeCell ref="B43:D43"/>
+    <mergeCell ref="B45:D45"/>
     <mergeCell ref="A33:E33"/>
     <mergeCell ref="A5:E5"/>
     <mergeCell ref="A23:E23"/>
     <mergeCell ref="A32:E32"/>
     <mergeCell ref="A8:E8"/>
     <mergeCell ref="A22:E22"/>
+    <mergeCell ref="B47:D47"/>
     <mergeCell ref="B17:E17"/>
     <mergeCell ref="A35:E35"/>
+    <mergeCell ref="B46:D46"/>
+    <mergeCell ref="A52:E52"/>
     <mergeCell ref="A10:E10"/>
     <mergeCell ref="A28:E28"/>
+    <mergeCell ref="A40:E40"/>
     <mergeCell ref="A13:E13"/>
     <mergeCell ref="B19:E19"/>
     <mergeCell ref="A31:E31"/>
     <mergeCell ref="A9:E9"/>
+    <mergeCell ref="B48:D48"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1256,6 +1323,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -1389,6 +1457,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
@@ -1480,6 +1549,7 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
@@ -1704,6 +1774,7 @@
         </is>
       </c>
     </row>
+    <row r="29"/>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
@@ -1814,7 +1885,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I176"/>
+  <dimension ref="A1:J176"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="66" customWidth="1" min="1" max="1"/>
@@ -1826,6 +1897,7 @@
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="62" customWidth="1" min="9" max="9"/>
+    <col width="80" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -1835,6 +1907,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="44" customHeight="1">
       <c r="A3" s="26" t="inlineStr">
         <is>
@@ -2000,6 +2073,7 @@
         <v/>
       </c>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="28" t="inlineStr">
         <is>
@@ -2038,6 +2112,16 @@
           <t>VERIF</t>
         </is>
       </c>
+      <c r="I20" s="35" t="inlineStr">
+        <is>
+          <t>Origem do valor (lista)</t>
+        </is>
+      </c>
+      <c r="J20" s="35" t="inlineStr">
+        <is>
+          <t>Fonte / observação</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -2103,7 +2187,7 @@
         <f>'09_LOADS'!$B$34</f>
         <v/>
       </c>
-      <c r="F22" s="20" t="n">
+      <c r="F22" s="16" t="n">
         <v>700</v>
       </c>
       <c r="G22" s="10" t="inlineStr">
@@ -2123,19 +2207,19 @@
           <t>Ângulo de deriva α (ISO 8855: + = velocidade p/ esquerda)</t>
         </is>
       </c>
-      <c r="B23" s="20" t="n">
+      <c r="B23" s="16" t="n">
         <v>-3</v>
       </c>
-      <c r="C23" s="20" t="n">
+      <c r="C23" s="16" t="n">
         <v>-3</v>
       </c>
-      <c r="D23" s="20" t="n">
+      <c r="D23" s="16" t="n">
         <v>-2</v>
       </c>
-      <c r="E23" s="20" t="n">
+      <c r="E23" s="16" t="n">
         <v>-2</v>
       </c>
-      <c r="F23" s="20" t="n">
+      <c r="F23" s="16" t="n">
         <v>3</v>
       </c>
       <c r="G23" s="10" t="inlineStr">
@@ -2146,6 +2230,16 @@
       <c r="H23" s="10" t="inlineStr">
         <is>
           <t>SUS-501</t>
+        </is>
+      </c>
+      <c r="I23" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
+      <c r="J23" s="45" t="inlineStr">
+        <is>
+          <t>Demonstrativos (EDR-022): α, γ e κ não vêm de cálculo do carro (não há modelo de slip). Valores arbitrários coerentes em sinal com 08_VEHICLE_STATE (curva à esquerda, frenagem). Substituir por casos de carga da equipe. VERIF (F): caso fixo de teste.</t>
         </is>
       </c>
     </row>
@@ -2155,19 +2249,19 @@
           <t>Camber γ (projeto: + = topo para fora)</t>
         </is>
       </c>
-      <c r="B24" s="20" t="n">
+      <c r="B24" s="16" t="n">
         <v>-1.5</v>
       </c>
-      <c r="C24" s="20" t="n">
+      <c r="C24" s="16" t="n">
         <v>-1.5</v>
       </c>
-      <c r="D24" s="20" t="n">
+      <c r="D24" s="16" t="n">
         <v>-1</v>
       </c>
-      <c r="E24" s="20" t="n">
+      <c r="E24" s="16" t="n">
         <v>-1</v>
       </c>
-      <c r="F24" s="20" t="n">
+      <c r="F24" s="16" t="n">
         <v>1.5</v>
       </c>
       <c r="G24" s="10" t="inlineStr">
@@ -2178,6 +2272,16 @@
       <c r="H24" s="10" t="inlineStr">
         <is>
           <t>SUS-404</t>
+        </is>
+      </c>
+      <c r="I24" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
+      <c r="J24" s="45" t="inlineStr">
+        <is>
+          <t>Camber de entrada manual (EDR-036 sem decisão: ainda não há ID para camber estático). Convenção do projeto: + = topo para fora, nos dois lados.</t>
         </is>
       </c>
     </row>
@@ -2187,19 +2291,19 @@
           <t>Slip ratio κ (ISO: −1 = travada em frenagem)</t>
         </is>
       </c>
-      <c r="B25" s="20" t="n">
+      <c r="B25" s="16" t="n">
         <v>-0.05</v>
       </c>
-      <c r="C25" s="20" t="n">
+      <c r="C25" s="16" t="n">
         <v>-0.05</v>
       </c>
-      <c r="D25" s="20" t="n">
+      <c r="D25" s="16" t="n">
         <v>-0.03</v>
       </c>
-      <c r="E25" s="20" t="n">
+      <c r="E25" s="16" t="n">
         <v>-0.03</v>
       </c>
-      <c r="F25" s="20" t="n">
+      <c r="F25" s="16" t="n">
         <v>0.05</v>
       </c>
       <c r="G25" s="10" t="inlineStr">
@@ -2210,6 +2314,16 @@
       <c r="H25" s="10" t="inlineStr">
         <is>
           <t>SUS-502</t>
+        </is>
+      </c>
+      <c r="I25" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
+      <c r="J25" s="45" t="inlineStr">
+        <is>
+          <t>Demonstrativo (EDR-022), como α e γ.</t>
         </is>
       </c>
     </row>
@@ -2245,6 +2359,7 @@
         </is>
       </c>
     </row>
+    <row r="27"/>
     <row r="28">
       <c r="A28" s="28" t="inlineStr">
         <is>
@@ -2415,6 +2530,7 @@
         </is>
       </c>
     </row>
+    <row r="33"/>
     <row r="34">
       <c r="A34" s="28" t="inlineStr">
         <is>
@@ -2644,6 +2760,7 @@
         </is>
       </c>
     </row>
+    <row r="41"/>
     <row r="42">
       <c r="A42" s="28" t="inlineStr">
         <is>
@@ -3021,6 +3138,7 @@
         </is>
       </c>
     </row>
+    <row r="53"/>
     <row r="54">
       <c r="A54" s="28" t="inlineStr">
         <is>
@@ -3435,6 +3553,7 @@
         </is>
       </c>
     </row>
+    <row r="66"/>
     <row r="67">
       <c r="A67" s="28" t="inlineStr">
         <is>
@@ -4031,6 +4150,18 @@
       <c r="H83" s="10" t="inlineStr">
         <is>
           <t>SUS-501</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="I84" s="10" t="inlineStr">
+        <is>
+          <t>◐ Provisório (.tir TTC)</t>
+        </is>
+      </c>
+      <c r="J84" s="45" t="inlineStr">
+        <is>
+          <t>Todos os coeficientes da tabela abaixo (B86:B175) foram transcritos do .tir provisório (ver os metadados acima). REFERENCE por natureza (DR-011), mas o dataset é provisório. Mudou o dataset: mudar o Tire REV (01_SETUP) e reexecutar 13_VALIDATION; os resultados antigos viram STALE.</t>
         </is>
       </c>
     </row>
@@ -6329,6 +6460,25 @@
     <mergeCell ref="A4:I4"/>
     <mergeCell ref="A54:I54"/>
   </mergeCells>
+  <conditionalFormatting sqref="I20:I176">
+    <cfRule type="expression" priority="1" dxfId="1">
+      <formula>LEFT($I20,1)="●"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="2">
+      <formula>LEFT($I20,1)="◐"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="3">
+      <formula>LEFT($I20,1)="○"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="4">
+      <formula>LEFT($I20,1)="?"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="I23 I24 I25 I84" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Origem fora da lista" error="Escolha uma das origens da lista (00_README, 'Como preencher')." type="list">
+      <formula1>=Origens</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
@@ -6340,14 +6490,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="80" customWidth="1" min="6" max="6"/>
+    <col hidden="1" width="13" customWidth="1" min="7" max="7"/>
+    <col hidden="1" width="13" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -6357,6 +6510,18 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Origem do valor (lista)</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Fonte / observação</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -6370,7 +6535,7 @@
           <t>Frequência-alvo dianteira</t>
         </is>
       </c>
-      <c r="B4" s="20" t="n">
+      <c r="B4" s="16" t="n">
         <v>2.5</v>
       </c>
       <c r="C4" s="10" t="inlineStr">
@@ -6381,6 +6546,24 @@
       <c r="D4" s="10" t="inlineStr">
         <is>
           <t>TARGET-001</t>
+        </is>
+      </c>
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
+      <c r="F4" s="45" t="inlineStr">
+        <is>
+          <t>Alvo demonstrativo: a meta da equipe está TBD em 03_TARGETS (TARGET-001).</t>
+        </is>
+      </c>
+      <c r="G4" s="10" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H4" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
         </is>
       </c>
     </row>
@@ -6390,7 +6573,7 @@
           <t>Frequência-alvo traseira</t>
         </is>
       </c>
-      <c r="B5" s="20" t="n">
+      <c r="B5" s="16" t="n">
         <v>2.7</v>
       </c>
       <c r="C5" s="10" t="inlineStr">
@@ -6403,7 +6586,26 @@
           <t>TARGET-002</t>
         </is>
       </c>
-    </row>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
+      <c r="F5" s="45" t="inlineStr">
+        <is>
+          <t>Alvo demonstrativo: a meta da equipe está TBD em 03_TARGETS (TARGET-002).</t>
+        </is>
+      </c>
+      <c r="G5" s="10" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="H5" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
+    </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
@@ -6495,6 +6697,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
@@ -6544,6 +6747,7 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
@@ -6557,7 +6761,7 @@
           <t>lambda_f alvo</t>
         </is>
       </c>
-      <c r="B18" s="20" t="n">
+      <c r="B18" s="16" t="n">
         <v>0.55</v>
       </c>
       <c r="C18" s="10" t="inlineStr">
@@ -6568,6 +6772,24 @@
       <c r="D18" s="10" t="inlineStr">
         <is>
           <t>TARGET-003</t>
+        </is>
+      </c>
+      <c r="E18" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
+      <c r="F18" s="45" t="inlineStr">
+        <is>
+          <t>Alvo demonstrativo: a meta da equipe está TBD em 03_TARGETS (TARGET-003).</t>
+        </is>
+      </c>
+      <c r="G18" s="10" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="H18" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
         </is>
       </c>
     </row>
@@ -6642,6 +6864,33 @@
     <mergeCell ref="A17:E17"/>
     <mergeCell ref="A3:E3"/>
   </mergeCells>
+  <conditionalFormatting sqref="E3:E21">
+    <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
+      <formula>AND(ISNUMBER($G3),$B3&lt;&gt;$G3,$E3=$H3)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="1">
+      <formula>LEFT($E3,1)="●"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="2">
+      <formula>LEFT($E3,1)="◐"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="5" dxfId="3">
+      <formula>LEFT($E3,1)="○"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="6" dxfId="4">
+      <formula>LEFT($E3,1)="?"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F3:F21">
+    <cfRule type="expression" priority="2" dxfId="5" stopIfTrue="1">
+      <formula>AND(LEFT($E3,1)="●",LEN(TRIM($F3))=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="E4 E5 E18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Origem fora da lista" error="Escolha uma das origens da lista (00_README, 'Como preencher')." type="list">
+      <formula1>=Origens</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
@@ -6670,6 +6919,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -6725,6 +6975,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -6837,6 +7088,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
@@ -6928,6 +7180,7 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
@@ -6998,6 +7251,7 @@
         </is>
       </c>
     </row>
+    <row r="20"/>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
@@ -7040,6 +7294,7 @@
         </is>
       </c>
     </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
@@ -7061,6 +7316,7 @@
         </is>
       </c>
     </row>
+    <row r="27"/>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
@@ -7159,6 +7415,7 @@
         </is>
       </c>
     </row>
+    <row r="34"/>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
@@ -7379,6 +7636,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -7407,6 +7665,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
@@ -7498,6 +7757,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
@@ -7610,6 +7870,7 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
@@ -7722,6 +7983,7 @@
         </is>
       </c>
     </row>
+    <row r="25"/>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
@@ -7813,6 +8075,7 @@
         </is>
       </c>
     </row>
+    <row r="31"/>
     <row r="32" ht="30" customHeight="1">
       <c r="A32" s="3" t="inlineStr">
         <is>
@@ -7967,7 +8230,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7984,6 +8247,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -8219,6 +8483,23 @@
       <c r="C16" s="12" t="inlineStr">
         <is>
           <t>Pedido do usuario (2026-10-19): seguir a literatura, principalmente o Milliken. EDR-045 a EDR-049. Registro celula a celula: docs/registro-de-versoes-V3_0.md. Validation: suspensao 54/54 (inclui exemplos da Milliken p. 683, p. 592, Tab. 16.3, Seward 4.1, Gillespie 5-8), Excel x Python (test_workbook e test_workbook_suspensao). NOT_VALIDATED fisicamente. Autor: nao registrado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>V3.0, 2a rodada (feedback da equipe): coluna Origem (lista) e Fonte em cada entrada (05, 06, 07, 08, 11; 10_TIRE I/J), com cores e aviso de origem desatualizada; fundo amarelo retirado e legenda corrigida; guia 'Como preencher' na 00_README.</t>
+        </is>
+      </c>
+      <c r="C17" s="12" t="inlineStr">
+        <is>
+          <t>Feedback da equipe (2026-10-14) e decisoes do usuario (2026-10-19). EDR-025 (A), EDR-035, EDR-051. Registro celula a celula: docs/registro-de-versoes-V3_0.md. Validation: test_workbook_suspensao (TC-WB30-010..012). NOT_VALIDATED fisicamente.</t>
         </is>
       </c>
     </row>
@@ -8253,6 +8534,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -8302,6 +8584,7 @@
       <c r="C6" s="10" t="inlineStr"/>
       <c r="D6" s="10" t="inlineStr"/>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
@@ -8402,6 +8685,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -8703,6 +8987,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="13" t="inlineStr">
         <is>
@@ -8753,6 +9038,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -8982,6 +9268,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="13" t="inlineStr">
         <is>
@@ -9033,6 +9320,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -9657,14 +9945,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="80" customWidth="1" min="6" max="6"/>
+    <col hidden="1" width="13" customWidth="1" min="7" max="7"/>
+    <col hidden="1" width="13" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -9674,6 +9965,18 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Origem do valor (lista)</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Fonte / observação</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -9700,6 +10003,24 @@
           <t>SUS-001</t>
         </is>
       </c>
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>○ Estimativa</t>
+        </is>
+      </c>
+      <c r="F4" s="45" t="inlineStr">
+        <is>
+          <t>Adesivo SAE Brasil 2026: 248,5 kg medidos sem piloto + 68 kg de piloto de referência (padrão FSAE, não medido). A célula mistura as duas origens: vale a pior.</t>
+        </is>
+      </c>
+      <c r="G4" s="10" t="n">
+        <v>316.5</v>
+      </c>
+      <c r="H4" s="10" t="inlineStr">
+        <is>
+          <t>○ Estimativa</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -9720,6 +10041,24 @@
           <t>SUS-002</t>
         </is>
       </c>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>● Dado do TX</t>
+        </is>
+      </c>
+      <c r="F5" s="45" t="inlineStr">
+        <is>
+          <t>E05, Key Parameters (315 mm). Medida a partir do plano do solo (SUS-000), não da origem do CAD.</t>
+        </is>
+      </c>
+      <c r="G5" s="10" t="n">
+        <v>0.315</v>
+      </c>
+      <c r="H5" s="10" t="inlineStr">
+        <is>
+          <t>● Dado do TX</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -9740,6 +10079,24 @@
           <t>SUS-003</t>
         </is>
       </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>● Dado do TX</t>
+        </is>
+      </c>
+      <c r="F6" s="45" t="inlineStr">
+        <is>
+          <t>E05, Key Parameters (1594 mm). Diverge do E03 (1550 mm, chassi anterior).</t>
+        </is>
+      </c>
+      <c r="G6" s="10" t="n">
+        <v>1.594</v>
+      </c>
+      <c r="H6" s="10" t="inlineStr">
+        <is>
+          <t>● Dado do TX</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -9760,6 +10117,24 @@
           <t>SUS-004</t>
         </is>
       </c>
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t>● Dado do TX</t>
+        </is>
+      </c>
+      <c r="F7" s="45" t="inlineStr">
+        <is>
+          <t>E05, Key Parameters (1277 mm).</t>
+        </is>
+      </c>
+      <c r="G7" s="10" t="n">
+        <v>1.277</v>
+      </c>
+      <c r="H7" s="10" t="inlineStr">
+        <is>
+          <t>● Dado do TX</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -9780,6 +10155,24 @@
           <t>SUS-005</t>
         </is>
       </c>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>● Dado do TX</t>
+        </is>
+      </c>
+      <c r="F8" s="45" t="inlineStr">
+        <is>
+          <t>E05, Key Parameters (1271 mm).</t>
+        </is>
+      </c>
+      <c r="G8" s="10" t="n">
+        <v>1.271</v>
+      </c>
+      <c r="H8" s="10" t="inlineStr">
+        <is>
+          <t>● Dado do TX</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -9800,6 +10193,24 @@
           <t>SUS-006</t>
         </is>
       </c>
+      <c r="E9" s="10" t="inlineStr">
+        <is>
+          <t>● Dado do TX</t>
+        </is>
+      </c>
+      <c r="F9" s="45" t="inlineStr">
+        <is>
+          <t>Derivado da distribuição medida no adesivo do TX/E05 (48,43 % no eixo dianteiro, com piloto) × wheelbase; coerente com a massa total, que inclui o piloto.</t>
+        </is>
+      </c>
+      <c r="G9" s="10" t="n">
+        <v>0.82203</v>
+      </c>
+      <c r="H9" s="10" t="inlineStr">
+        <is>
+          <t>● Dado do TX</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -9820,6 +10231,24 @@
           <t>SUS-006</t>
         </is>
       </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>● Dado do TX</t>
+        </is>
+      </c>
+      <c r="F10" s="45" t="inlineStr">
+        <is>
+          <t>Derivado da distribuição medida no adesivo do TX/E05 (51,57 % no eixo traseiro, com piloto) × wheelbase.</t>
+        </is>
+      </c>
+      <c r="G10" s="10" t="n">
+        <v>0.77197</v>
+      </c>
+      <c r="H10" s="10" t="inlineStr">
+        <is>
+          <t>● Dado do TX</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="18" t="inlineStr">
@@ -9832,6 +10261,7 @@
         <v/>
       </c>
     </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
@@ -9858,6 +10288,24 @@
           <t>SUS-007</t>
         </is>
       </c>
+      <c r="E14" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
+      <c r="F14" s="45" t="inlineStr">
+        <is>
+          <t>Não disponível para o TX/E05: a pesagem em plataforma mede a carga total no solo e não separa massa suspensa de não suspensa (confirmado pela equipe). Valor arbitrário: não usar para decisão de projeto.</t>
+        </is>
+      </c>
+      <c r="G14" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="H14" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -9878,6 +10326,24 @@
           <t>SUS-008</t>
         </is>
       </c>
+      <c r="E15" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
+      <c r="F15" s="45" t="inlineStr">
+        <is>
+          <t>Não disponível para o TX/E05 (mesma razão do SUS-007). Valor arbitrário: não usar para decisão de projeto.</t>
+        </is>
+      </c>
+      <c r="G15" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="H15" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -9898,6 +10364,24 @@
           <t>SUS-010</t>
         </is>
       </c>
+      <c r="E16" s="10" t="inlineStr">
+        <is>
+          <t>○ Estimativa</t>
+        </is>
+      </c>
+      <c r="F16" s="45" t="inlineStr">
+        <is>
+          <t>Estimativa pelo raio do pneu 20.0-13 do E03 (diâmetro 20,0 in / 2 = 0,254 m); não é medição da equipe.</t>
+        </is>
+      </c>
+      <c r="G16" s="10" t="n">
+        <v>0.254</v>
+      </c>
+      <c r="H16" s="10" t="inlineStr">
+        <is>
+          <t>○ Estimativa</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -9918,7 +10402,26 @@
           <t>SUS-011</t>
         </is>
       </c>
-    </row>
+      <c r="E17" s="10" t="inlineStr">
+        <is>
+          <t>○ Estimativa</t>
+        </is>
+      </c>
+      <c r="F17" s="45" t="inlineStr">
+        <is>
+          <t>Estimativa pelo raio do pneu 20.0-13 do E03 (mesmo pneu na frente e atrás); não é medição da equipe.</t>
+        </is>
+      </c>
+      <c r="G17" s="10" t="n">
+        <v>0.254</v>
+      </c>
+      <c r="H17" s="10" t="inlineStr">
+        <is>
+          <t>○ Estimativa</t>
+        </is>
+      </c>
+    </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
@@ -9932,7 +10435,7 @@
           <t>Ground Plane Z (offset origem CAD -&gt; solo)</t>
         </is>
       </c>
-      <c r="B20" s="20" t="n">
+      <c r="B20" s="16" t="n">
         <v>-0.05</v>
       </c>
       <c r="C20" s="10" t="inlineStr">
@@ -9945,7 +10448,26 @@
           <t>SUS-000</t>
         </is>
       </c>
-    </row>
+      <c r="E20" s="10" t="inlineStr">
+        <is>
+          <t>? A confirmar</t>
+        </is>
+      </c>
+      <c r="F20" s="45" t="inlineStr">
+        <is>
+          <t>SUS-000: coordenada Z do solo no sistema de coordenadas da equipe. As alturas desta planilha já são medidas a partir do solo (ficha SUS-000 do Engineering Standard). A origem do valor −0,05 m não está registrada.</t>
+        </is>
+      </c>
+      <c r="G20" s="10" t="n">
+        <v>-0.05</v>
+      </c>
+      <c r="H20" s="10" t="inlineStr">
+        <is>
+          <t>? A confirmar</t>
+        </is>
+      </c>
+    </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
@@ -10066,6 +10588,33 @@
     <mergeCell ref="A22:E22"/>
     <mergeCell ref="A3:E3"/>
   </mergeCells>
+  <conditionalFormatting sqref="E3:E27">
+    <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
+      <formula>AND(ISNUMBER($G3),$B3&lt;&gt;$G3,$E3=$H3)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="1">
+      <formula>LEFT($E3,1)="●"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="2">
+      <formula>LEFT($E3,1)="◐"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="5" dxfId="3">
+      <formula>LEFT($E3,1)="○"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="6" dxfId="4">
+      <formula>LEFT($E3,1)="?"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F3:F27">
+    <cfRule type="expression" priority="2" dxfId="5" stopIfTrue="1">
+      <formula>AND(LEFT($E3,1)="●",LEN(TRIM($F3))=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="E4 E5 E6 E7 E8 E9 E10 E14 E15 E16 E17 E20" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Origem fora da lista" error="Escolha uma das origens da lista (00_README, 'Como preencher')." type="list">
+      <formula1>=Origens</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
@@ -10077,14 +10626,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:H52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="80" customWidth="1" min="6" max="6"/>
+    <col hidden="1" width="13" customWidth="1" min="7" max="7"/>
+    <col hidden="1" width="13" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -10100,6 +10652,16 @@
           <t>Mola, MR, barra e roll center (B4:B15): valores DEMONSTRATIVOS herdados do T09/E03, para referência e teste das fórmulas; não são o TX/E05 (EDR-012/022).</t>
         </is>
       </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Origem do valor (lista)</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Fonte / observação</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -10127,6 +10689,24 @@
           <t>SUS-203</t>
         </is>
       </c>
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>◐ Dado do T09</t>
+        </is>
+      </c>
+      <c r="F4" s="45" t="inlineStr">
+        <is>
+          <t>Demonstrativo (EDR-012/022): valor do T09/E03 para referência, comparação e teste das fórmulas (usuário, 2026-10-19); não é o TX/E05. Calculado a partir da planilha detalhada do T09: ride rate dianteiro 16 112,23 N/m (que é o wheel rate) × MR² (MR = 1,76). Corrige o valor anterior, do spec sheet resumido, que arredondava F e R como iguais.</t>
+        </is>
+      </c>
+      <c r="G4" s="10" t="n">
+        <v>49909.24</v>
+      </c>
+      <c r="H4" s="10" t="inlineStr">
+        <is>
+          <t>◐ Dado do T09</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -10147,6 +10727,24 @@
           <t>SUS-203</t>
         </is>
       </c>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>◐ Dado do T09</t>
+        </is>
+      </c>
+      <c r="F5" s="45" t="inlineStr">
+        <is>
+          <t>Demonstrativo (EDR-012/022): valor do T09/E03 para referência, comparação e teste das fórmulas (usuário, 2026-10-19); não é o TX/E05. Calculado a partir da planilha detalhada do T09: ride rate traseiro 18 418,2 N/m × MR² (MR = 1,76).</t>
+        </is>
+      </c>
+      <c r="G5" s="10" t="n">
+        <v>57052.22</v>
+      </c>
+      <c r="H5" s="10" t="inlineStr">
+        <is>
+          <t>◐ Dado do T09</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -10167,6 +10765,24 @@
           <t>SUS-201</t>
         </is>
       </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>◐ Dado do T09</t>
+        </is>
+      </c>
+      <c r="F6" s="45" t="inlineStr">
+        <is>
+          <t>Demonstrativo (EDR-012/022): valor do T09/E03 para referência, comparação e teste das fórmulas (usuário, 2026-10-19); não é o TX/E05. E03 (1,76:1). Convenção wheel/spring assumida (igual à do projeto); o E03 não diz a direção.</t>
+        </is>
+      </c>
+      <c r="G6" s="10" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="H6" s="10" t="inlineStr">
+        <is>
+          <t>◐ Dado do T09</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -10187,7 +10803,26 @@
           <t>SUS-201</t>
         </is>
       </c>
-    </row>
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t>◐ Dado do T09</t>
+        </is>
+      </c>
+      <c r="F7" s="45" t="inlineStr">
+        <is>
+          <t>Demonstrativo (EDR-012/022): valor do T09/E03 para referência, comparação e teste das fórmulas (usuário, 2026-10-19); não é o TX/E05. E03 (1,76:1, igual à dianteira).</t>
+        </is>
+      </c>
+      <c r="G7" s="10" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="H7" s="10" t="inlineStr">
+        <is>
+          <t>◐ Dado do T09</t>
+        </is>
+      </c>
+    </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
@@ -10214,6 +10849,24 @@
           <t>SUS-206</t>
         </is>
       </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>◐ Dado do T09</t>
+        </is>
+      </c>
+      <c r="F10" s="45" t="inlineStr">
+        <is>
+          <t>Demonstrativo (EDR-012/022): valor do T09/E03 para referência, comparação e teste das fórmulas (usuário, 2026-10-19); não é o TX/E05. Planilha detalhada do T09 (AntiRoll Bar Rate dianteiro), valor direto.</t>
+        </is>
+      </c>
+      <c r="G10" s="10" t="n">
+        <v>5012.32</v>
+      </c>
+      <c r="H10" s="10" t="inlineStr">
+        <is>
+          <t>◐ Dado do T09</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -10234,7 +10887,26 @@
           <t>SUS-207</t>
         </is>
       </c>
-    </row>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>◐ Dado do T09</t>
+        </is>
+      </c>
+      <c r="F11" s="45" t="inlineStr">
+        <is>
+          <t>Demonstrativo (EDR-012/022): valor do T09/E03 para referência, comparação e teste das fórmulas (usuário, 2026-10-19); não é o TX/E05. Planilha detalhada do T09 (AntiRoll Bar Rate traseiro, ≈ 0, coerente com 'sem ARB').</t>
+        </is>
+      </c>
+      <c r="G11" s="10" t="n">
+        <v>10.78</v>
+      </c>
+      <c r="H11" s="10" t="inlineStr">
+        <is>
+          <t>◐ Dado do T09</t>
+        </is>
+      </c>
+    </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
@@ -10261,6 +10933,24 @@
           <t>SUS-401-F</t>
         </is>
       </c>
+      <c r="E14" s="10" t="inlineStr">
+        <is>
+          <t>◐ Dado do T09</t>
+        </is>
+      </c>
+      <c r="F14" s="45" t="inlineStr">
+        <is>
+          <t>Demonstrativo (EDR-012/022): valor do T09/E03 para referência, comparação e teste das fórmulas (usuário, 2026-10-19); não é o TX/E05. Planilha detalhada do T09 (0,0675 m), mais precisa que o spec sheet do E03 (60 mm, arredondado). Provisório até a Fase 2 (OptimumKinematics).</t>
+        </is>
+      </c>
+      <c r="G14" s="10" t="n">
+        <v>0.0675</v>
+      </c>
+      <c r="H14" s="10" t="inlineStr">
+        <is>
+          <t>◐ Dado do T09</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -10281,7 +10971,26 @@
           <t>SUS-401-R</t>
         </is>
       </c>
-    </row>
+      <c r="E15" s="10" t="inlineStr">
+        <is>
+          <t>◐ Dado do T09</t>
+        </is>
+      </c>
+      <c r="F15" s="45" t="inlineStr">
+        <is>
+          <t>Demonstrativo (EDR-012/022): valor do T09/E03 para referência, comparação e teste das fórmulas (usuário, 2026-10-19); não é o TX/E05. E03 (110 mm, roll center estático acima do solo). Provisório até a Fase 2 (OptimumKinematics).</t>
+        </is>
+      </c>
+      <c r="G15" s="10" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="H15" s="10" t="inlineStr">
+        <is>
+          <t>◐ Dado do T09</t>
+        </is>
+      </c>
+    </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
@@ -10457,6 +11166,7 @@
         </is>
       </c>
     </row>
+    <row r="26"/>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
@@ -10506,6 +11216,7 @@
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
@@ -10575,7 +11286,7 @@
           <t>Front Brake Force Fraction (FB_f)</t>
         </is>
       </c>
-      <c r="B36" s="20" t="n">
+      <c r="B36" s="16" t="n">
         <v>0.6</v>
       </c>
       <c r="C36" s="10" t="inlineStr">
@@ -10586,6 +11297,24 @@
       <c r="D36" s="10" t="inlineStr">
         <is>
           <t>SUS-013</t>
+        </is>
+      </c>
+      <c r="E36" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
+      <c r="F36" s="45" t="inlineStr">
+        <is>
+          <t>Placeholder: fração da força de frenagem no eixo dianteiro (brake bias). Substituir pelo balanço de freio real do Setup.</t>
+        </is>
+      </c>
+      <c r="G36" s="10" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H36" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
         </is>
       </c>
     </row>
@@ -10608,6 +11337,24 @@
           <t>SUS-014</t>
         </is>
       </c>
+      <c r="E37" s="10" t="inlineStr">
+        <is>
+          <t>○ Estimativa</t>
+        </is>
+      </c>
+      <c r="F37" s="45" t="inlineStr">
+        <is>
+          <t>Hipótese congelada da V1: TF_r = 1 (tração só traseira). Revisitar se a equipe mudar para AWD.</t>
+        </is>
+      </c>
+      <c r="G37" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H37" s="10" t="inlineStr">
+        <is>
+          <t>○ Estimativa</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
@@ -10693,6 +11440,7 @@
         </is>
       </c>
     </row>
+    <row r="42"/>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
@@ -10706,7 +11454,7 @@
           <t>Steering Ratio (SR)</t>
         </is>
       </c>
-      <c r="B44" s="20" t="n">
+      <c r="B44" s="16" t="n">
         <v>4.5</v>
       </c>
       <c r="C44" s="10" t="inlineStr">
@@ -10719,7 +11467,26 @@
           <t>SUS-601</t>
         </is>
       </c>
-    </row>
+      <c r="E44" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
+      <c r="F44" s="45" t="inlineStr">
+        <is>
+          <t>Placeholder: razão entre o ângulo do volante e o ângulo médio das rodas dianteiras. Substituir pela medição da cremalheira ou pela geometria do rack.</t>
+        </is>
+      </c>
+      <c r="G44" s="10" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H44" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
+    </row>
+    <row r="45"/>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
@@ -10746,6 +11513,24 @@
           <t>SUS-211</t>
         </is>
       </c>
+      <c r="E47" s="10" t="inlineStr">
+        <is>
+          <t>◐ Provisório (.tir TTC)</t>
+        </is>
+      </c>
+      <c r="F47" s="45" t="inlineStr">
+        <is>
+          <t>VERTICAL_STIFFNESS do .tir TTC provisório (Hoosier R25B; EDR-038, EDR-045). Não é o pneu do carro nem medição da equipe: substituir pela rigidez vertical do pneu real.</t>
+        </is>
+      </c>
+      <c r="G47" s="10" t="n">
+        <v>120312</v>
+      </c>
+      <c r="H47" s="10" t="inlineStr">
+        <is>
+          <t>◐ Provisório (.tir TTC)</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
@@ -10764,6 +11549,24 @@
       <c r="D48" s="10" t="inlineStr">
         <is>
           <t>SUS-211</t>
+        </is>
+      </c>
+      <c r="E48" s="10" t="inlineStr">
+        <is>
+          <t>◐ Provisório (.tir TTC)</t>
+        </is>
+      </c>
+      <c r="F48" s="45" t="inlineStr">
+        <is>
+          <t>VERTICAL_STIFFNESS do .tir TTC provisório (Hoosier R25B; EDR-038, EDR-045). Não é o pneu do carro nem medição da equipe: substituir pela rigidez vertical do pneu real.</t>
+        </is>
+      </c>
+      <c r="G48" s="10" t="n">
+        <v>120312</v>
+      </c>
+      <c r="H48" s="10" t="inlineStr">
+        <is>
+          <t>◐ Provisório (.tir TTC)</t>
         </is>
       </c>
     </row>
@@ -10864,6 +11667,33 @@
     <mergeCell ref="A27:E27"/>
     <mergeCell ref="A3:E3"/>
   </mergeCells>
+  <conditionalFormatting sqref="E3:E52">
+    <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
+      <formula>AND(ISNUMBER($G3),$B3&lt;&gt;$G3,$E3=$H3)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="1">
+      <formula>LEFT($E3,1)="●"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="2">
+      <formula>LEFT($E3,1)="◐"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="5" dxfId="3">
+      <formula>LEFT($E3,1)="○"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="6" dxfId="4">
+      <formula>LEFT($E3,1)="?"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F3:F52">
+    <cfRule type="expression" priority="2" dxfId="5" stopIfTrue="1">
+      <formula>AND(LEFT($E3,1)="●",LEN(TRIM($F3))=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="E4 E5 E6 E7 E10 E11 E14 E15 E36 E37 E44 E47 E48" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Origem fora da lista" error="Escolha uma das origens da lista (00_README, 'Como preencher')." type="list">
+      <formula1>=Origens</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
@@ -10875,14 +11705,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E69"/>
+  <dimension ref="A1:H69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="80" customWidth="1" min="6" max="6"/>
+    <col hidden="1" width="13" customWidth="1" min="7" max="7"/>
+    <col hidden="1" width="13" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -10892,6 +11725,18 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Origem do valor (lista)</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Fonte / observação</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -10906,6 +11751,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
@@ -10935,6 +11781,7 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
@@ -10961,6 +11808,24 @@
           <t>SUS-406-F</t>
         </is>
       </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
+      <c r="F10" s="45" t="inlineStr">
+        <is>
+          <t>Placeholder geométrico para testar a fórmula; não é hardpoint real. Fase 2: REFERENCE do OptimumKinematics.</t>
+        </is>
+      </c>
+      <c r="G10" s="10" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H10" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -10981,6 +11846,24 @@
           <t>SUS-406-F</t>
         </is>
       </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
+      <c r="F11" s="45" t="inlineStr">
+        <is>
+          <t>Placeholder geométrico (07_KINEMATICS inteira é placeholder até a Fase 2); não é hardpoint real.</t>
+        </is>
+      </c>
+      <c r="G11" s="10" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="H11" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -11001,6 +11884,24 @@
           <t>SUS-406-R</t>
         </is>
       </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
+      <c r="F12" s="45" t="inlineStr">
+        <is>
+          <t>Placeholder geométrico (07_KINEMATICS inteira é placeholder até a Fase 2); não é hardpoint real.</t>
+        </is>
+      </c>
+      <c r="G12" s="10" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="H12" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -11021,6 +11922,24 @@
           <t>SUS-406-R</t>
         </is>
       </c>
+      <c r="E13" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
+      <c r="F13" s="45" t="inlineStr">
+        <is>
+          <t>Placeholder geométrico (07_KINEMATICS inteira é placeholder até a Fase 2); não é hardpoint real.</t>
+        </is>
+      </c>
+      <c r="G13" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="H13" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -11042,6 +11961,11 @@
           <t>SUS-406-R</t>
         </is>
       </c>
+      <c r="F14" s="45" t="inlineStr">
+        <is>
+          <t>Calculada: = SUS-011 (05_VEHICLE B17). Placeholder: substituir pela altura do centro da roda do CAD.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -11076,6 +12000,24 @@
           <t>SUS-403-F</t>
         </is>
       </c>
+      <c r="E17" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
+      <c r="F17" s="45" t="inlineStr">
+        <is>
+          <t>Placeholder geométrico (07_KINEMATICS inteira é placeholder até a Fase 2); não é hardpoint real.</t>
+        </is>
+      </c>
+      <c r="G17" s="10" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H17" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -11096,6 +12038,24 @@
           <t>SUS-403-F</t>
         </is>
       </c>
+      <c r="E18" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
+      <c r="F18" s="45" t="inlineStr">
+        <is>
+          <t>Placeholder geométrico (07_KINEMATICS inteira é placeholder até a Fase 2); não é hardpoint real.</t>
+        </is>
+      </c>
+      <c r="G18" s="10" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H18" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -11116,6 +12076,24 @@
           <t>SUS-403-R</t>
         </is>
       </c>
+      <c r="E19" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
+      <c r="F19" s="45" t="inlineStr">
+        <is>
+          <t>Placeholder geométrico (07_KINEMATICS inteira é placeholder até a Fase 2); não é hardpoint real.</t>
+        </is>
+      </c>
+      <c r="G19" s="10" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="H19" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -11136,7 +12114,26 @@
           <t>SUS-403-R</t>
         </is>
       </c>
-    </row>
+      <c r="E20" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
+      <c r="F20" s="45" t="inlineStr">
+        <is>
+          <t>Placeholder geométrico (07_KINEMATICS inteira é placeholder até a Fase 2); não é hardpoint real.</t>
+        </is>
+      </c>
+      <c r="G20" s="10" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H20" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
+    </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
@@ -11163,6 +12160,24 @@
           <t>SUS-404-F</t>
         </is>
       </c>
+      <c r="E23" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
+      <c r="F23" s="45" t="inlineStr">
+        <is>
+          <t>Placeholder geométrico (07_KINEMATICS inteira é placeholder até a Fase 2); não é hardpoint real.</t>
+        </is>
+      </c>
+      <c r="G23" s="10" t="n">
+        <v>-0.6</v>
+      </c>
+      <c r="H23" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -11183,7 +12198,26 @@
           <t>SUS-404-R</t>
         </is>
       </c>
-    </row>
+      <c r="E24" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
+      <c r="F24" s="45" t="inlineStr">
+        <is>
+          <t>Placeholder geométrico (07_KINEMATICS inteira é placeholder até a Fase 2); não é hardpoint real.</t>
+        </is>
+      </c>
+      <c r="G24" s="10" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="H24" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
+    </row>
+    <row r="25"/>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
@@ -11210,6 +12244,24 @@
           <t>SUS-405-F</t>
         </is>
       </c>
+      <c r="E27" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
+      <c r="F27" s="45" t="inlineStr">
+        <is>
+          <t>Placeholder geométrico (07_KINEMATICS inteira é placeholder até a Fase 2); não é hardpoint real.</t>
+        </is>
+      </c>
+      <c r="G27" s="10" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="H27" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -11230,7 +12282,26 @@
           <t>SUS-405-R</t>
         </is>
       </c>
-    </row>
+      <c r="E28" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
+      <c r="F28" s="45" t="inlineStr">
+        <is>
+          <t>Placeholder geométrico (07_KINEMATICS inteira é placeholder até a Fase 2); não é hardpoint real.</t>
+        </is>
+      </c>
+      <c r="G28" s="10" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="H28" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
+    </row>
+    <row r="29"/>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
@@ -11257,6 +12328,24 @@
           <t>-</t>
         </is>
       </c>
+      <c r="E31" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
+      <c r="F31" s="45" t="inlineStr">
+        <is>
+          <t>Placeholder geométrico; não é a medição do curso instalado. Substituir pelo curso real (bump + rebound) com o piloto sentado, conforme V.3.1.1.</t>
+        </is>
+      </c>
+      <c r="G31" s="10" t="n">
+        <v>60</v>
+      </c>
+      <c r="H31" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -11277,7 +12366,26 @@
           <t>-</t>
         </is>
       </c>
-    </row>
+      <c r="E32" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
+      <c r="F32" s="45" t="inlineStr">
+        <is>
+          <t>Placeholder geométrico; não é a medição do curso instalado (ver B31).</t>
+        </is>
+      </c>
+      <c r="G32" s="10" t="n">
+        <v>65</v>
+      </c>
+      <c r="H32" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
+    </row>
+    <row r="33"/>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
@@ -11994,6 +13102,7 @@
         </is>
       </c>
     </row>
+    <row r="62"/>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
@@ -12149,6 +13258,33 @@
     <mergeCell ref="A9:E9"/>
     <mergeCell ref="A3:E3"/>
   </mergeCells>
+  <conditionalFormatting sqref="E3:E69">
+    <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
+      <formula>AND(ISNUMBER($G3),$B3&lt;&gt;$G3,$E3=$H3)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="1">
+      <formula>LEFT($E3,1)="●"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="2">
+      <formula>LEFT($E3,1)="◐"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="5" dxfId="3">
+      <formula>LEFT($E3,1)="○"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="6" dxfId="4">
+      <formula>LEFT($E3,1)="?"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F3:F69">
+    <cfRule type="expression" priority="2" dxfId="5" stopIfTrue="1">
+      <formula>AND(LEFT($E3,1)="●",LEN(TRIM($F3))=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="E10 E11 E12 E13 E17 E18 E19 E20 E23 E24 E27 E28 E31 E32" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Origem fora da lista" error="Escolha uma das origens da lista (00_README, 'Como preencher')." type="list">
+      <formula1>=Origens</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
@@ -12160,14 +13296,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="80" customWidth="1" min="6" max="6"/>
+    <col hidden="1" width="13" customWidth="1" min="7" max="7"/>
+    <col hidden="1" width="13" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -12177,6 +13316,18 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Origem do valor (lista)</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Fonte / observação</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -12203,6 +13354,24 @@
           <t>-</t>
         </is>
       </c>
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>○ Estimativa</t>
+        </is>
+      </c>
+      <c r="F4" s="45" t="inlineStr">
+        <is>
+          <t>Caso de carga sem fonte registrada. ISO 8855: a_x + = aceleração para frente (transfere carga para o eixo traseiro); negativo = frenagem.</t>
+        </is>
+      </c>
+      <c r="G4" s="10" t="n">
+        <v>-5</v>
+      </c>
+      <c r="H4" s="10" t="inlineStr">
+        <is>
+          <t>○ Estimativa</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -12223,7 +13392,26 @@
           <t>-</t>
         </is>
       </c>
-    </row>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>○ Estimativa</t>
+        </is>
+      </c>
+      <c r="F5" s="45" t="inlineStr">
+        <is>
+          <t>Caso de carga sem fonte registrada. Curva à esquerda de 1,2 g. ISO 8855: a_y + = para a esquerda (o lado direito ganha carga).</t>
+        </is>
+      </c>
+      <c r="G5" s="10" t="n">
+        <v>11.772</v>
+      </c>
+      <c r="H5" s="10" t="inlineStr">
+        <is>
+          <t>○ Estimativa</t>
+        </is>
+      </c>
+    </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
@@ -12250,6 +13438,24 @@
           <t>SUS-701</t>
         </is>
       </c>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>○ Estimativa</t>
+        </is>
+      </c>
+      <c r="F8" s="45" t="inlineStr">
+        <is>
+          <t>Caso de carga sem fonte registrada. Aero constante por Setup (SUS-701, EDR-013).</t>
+        </is>
+      </c>
+      <c r="G8" s="10" t="n">
+        <v>400</v>
+      </c>
+      <c r="H8" s="10" t="inlineStr">
+        <is>
+          <t>○ Estimativa</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -12268,6 +13474,24 @@
       <c r="D9" s="10" t="inlineStr">
         <is>
           <t>SUS-702</t>
+        </is>
+      </c>
+      <c r="E9" s="10" t="inlineStr">
+        <is>
+          <t>○ Estimativa</t>
+        </is>
+      </c>
+      <c r="F9" s="45" t="inlineStr">
+        <is>
+          <t>Caso de carga sem fonte registrada. Fração dianteira da downforce (SUS-702, EDR-013).</t>
+        </is>
+      </c>
+      <c r="G9" s="10" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="H9" s="10" t="inlineStr">
+        <is>
+          <t>○ Estimativa</t>
         </is>
       </c>
     </row>
@@ -12277,7 +13501,33 @@
     <mergeCell ref="A7:E7"/>
     <mergeCell ref="A3:E3"/>
   </mergeCells>
+  <conditionalFormatting sqref="E3:E9">
+    <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
+      <formula>AND(ISNUMBER($G3),$B3&lt;&gt;$G3,$E3=$H3)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="1">
+      <formula>LEFT($E3,1)="●"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="2">
+      <formula>LEFT($E3,1)="◐"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="5" dxfId="3">
+      <formula>LEFT($E3,1)="○"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="6" dxfId="4">
+      <formula>LEFT($E3,1)="?"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F3:F9">
+    <cfRule type="expression" priority="2" dxfId="5" stopIfTrue="1">
+      <formula>AND(LEFT($E3,1)="●",LEN(TRIM($F3))=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="E4 E5 E8 E9" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Origem fora da lista" error="Escolha uma das origens da lista (00_README, 'Como preencher')." type="list">
+      <formula1>=Origens</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: valores derivados da planilha V3.0 viram fórmula (FB-05, EDR-050)
Feedback da equipe: números calculados estavam digitados. Regra do
usuário: com parcela externa, a parcela vira entrada (com origem) e a
célula vira a conta.

- 05_VEHICLE: entradas novas B30 (massa medida sem piloto), B31 (piloto),
  B32 (fração de peso dianteira), B33/B34 (diâmetro do pneu); B4, B9,
  B10, B16 e B17 passam a ser fórmula.
- 08_VEHICLE_STATE: B11 (a_y em g) e B5 = B11*9.81.
- Efeito: só o arredondamento antigo de a e b (Fz muda <= 0,005 N).
- 356 -> 362 fórmulas; TC-WB30-013; TC-WB30-002/005/006 escrevem as
  parcelas. Suíte inteira PASS; test_workbook_suspensao 13/13 pelo Excel
  e pelo LibreOffice.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel/FSAE_EV_Suspension_Fase1_V3_0.xlsx
+++ b/excel/FSAE_EV_Suspension_Fase1_V3_0.xlsx
@@ -846,7 +846,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Versão do workbook: V3.0 (em desenvolvimento até concluir as correções de feedback; revisão metodológica contra Milliken/Gillespie/Seward/Pacejka: pneu em série, termo gravitacional da rolagem, massa suspensa por eixo, anti com sinal, Ky com um λFz0; EDR-045 a EDR-049; 2ª rodada, feedback da equipe: origem de cada entrada, guia de preenchimento; EDR-035, EDR-051) | Status: DRAFT — cross-check, ainda NÃO REFERENCE-validated</t>
+          <t>Versão do workbook: V3.0 (em desenvolvimento até concluir as correções de feedback; revisão metodológica contra Milliken/Gillespie/Seward/Pacejka: pneu em série, termo gravitacional da rolagem, massa suspensa por eixo, anti com sinal, Ky com um λFz0; EDR-045 a EDR-049; 2ª rodada, feedback da equipe: origem de cada entrada, valores derivados como fórmula, guia de preenchimento; EDR-035, EDR-050, EDR-051) | Status: DRAFT — cross-check, ainda NÃO REFERENCE-validated</t>
         </is>
       </c>
     </row>
@@ -1089,7 +1089,7 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>Como preencher esta planilha (EDR-035, EDR-051)</t>
+          <t>Como preencher esta planilha (EDR-035, EDR-050, EDR-051)</t>
         </is>
       </c>
     </row>
@@ -1236,18 +1236,24 @@
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>4. Até a V3.0 ser fechada, esta planilha é gerada pelo script do repositório e o que for digitado nela se perde na próxima geração (EDR-051). Depois do fechamento, ela passa a ser o arquivo da equipe.</t>
+          <t>4. Valor que sai de conta não é digitado (EDR-050): digite as parcelas, não o resultado. Exemplo: massa total = massa medida + piloto (05_VEHICLE B30 e B31).</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>5. Convenções de sinais e eixos: seção acima. Decisões e fichas: pasta docs/ do repositório (Engineering_Decision_Register.md e Engineering Standard).</t>
-        </is>
-      </c>
-    </row>
-    <row r="52"/>
+          <t>5. Até a V3.0 ser fechada, esta planilha é gerada pelo script do repositório e o que for digitado nela se perde na próxima geração (EDR-051). Depois do fechamento, ela passa a ser o arquivo da equipe.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>6. Convenções de sinais e eixos: seção acima. Decisões e fichas: pasta docs/ do repositório (Engineering_Decision_Register.md e Engineering Standard).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="45">
     <mergeCell ref="A30:E30"/>
@@ -8494,12 +8500,12 @@
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>V3.0, 2a rodada (feedback da equipe): coluna Origem (lista) e Fonte em cada entrada (05, 06, 07, 08, 11; 10_TIRE I/J), com cores e aviso de origem desatualizada; fundo amarelo retirado e legenda corrigida; guia 'Como preencher' na 00_README.</t>
+          <t>V3.0, 2a rodada (feedback da equipe): coluna Origem (lista) e Fonte em cada entrada (05, 06, 07, 08, 11; 10_TIRE I/J), com cores e aviso de origem desatualizada; fundo amarelo retirado e legenda corrigida; valores derivados como formula (05_VEHICLE B4, B9, B10, B16, B17; 08 B5; entradas novas 05 B30:B34 e 08 B11); guia 'Como preencher' na 00_README.</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>Feedback da equipe (2026-10-14) e decisoes do usuario (2026-10-19). EDR-025 (A), EDR-035, EDR-051. Registro celula a celula: docs/registro-de-versoes-V3_0.md. Validation: test_workbook_suspensao (TC-WB30-010..012). NOT_VALIDATED fisicamente.</t>
+          <t>Feedback da equipe (2026-10-14) e decisoes do usuario (2026-10-19). EDR-025 (A), EDR-035, EDR-050, EDR-051. Registro celula a celula: docs/registro-de-versoes-V3_0.md. Validation: test_workbook_suspensao (TC-WB30-010..013). NOT_VALIDATED fisicamente.</t>
         </is>
       </c>
     </row>
@@ -9945,7 +9951,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -9990,8 +9996,9 @@
           <t>Massa total (com piloto)</t>
         </is>
       </c>
-      <c r="B4" s="16" t="n">
-        <v>316.5</v>
+      <c r="B4" s="21">
+        <f>'05_VEHICLE'!$B$30+'05_VEHICLE'!$B$31</f>
+        <v/>
       </c>
       <c r="C4" s="10" t="inlineStr">
         <is>
@@ -10003,22 +10010,9 @@
           <t>SUS-001</t>
         </is>
       </c>
-      <c r="E4" s="10" t="inlineStr">
-        <is>
-          <t>○ Estimativa</t>
-        </is>
-      </c>
       <c r="F4" s="45" t="inlineStr">
         <is>
-          <t>Adesivo SAE Brasil 2026: 248,5 kg medidos sem piloto + 68 kg de piloto de referência (padrão FSAE, não medido). A célula mistura as duas origens: vale a pior.</t>
-        </is>
-      </c>
-      <c r="G4" s="10" t="n">
-        <v>316.5</v>
-      </c>
-      <c r="H4" s="10" t="inlineStr">
-        <is>
-          <t>○ Estimativa</t>
+          <t>Calculada (EDR-050): massa medida sem piloto (B30) + massa do piloto (B31).</t>
         </is>
       </c>
     </row>
@@ -10180,8 +10174,9 @@
           <t>CG -&gt; eixo dianteiro (a)</t>
         </is>
       </c>
-      <c r="B9" s="16" t="n">
-        <v>0.82203</v>
+      <c r="B9" s="21">
+        <f>'05_VEHICLE'!$B$6*(1-'05_VEHICLE'!$B$32)</f>
+        <v/>
       </c>
       <c r="C9" s="10" t="inlineStr">
         <is>
@@ -10193,22 +10188,9 @@
           <t>SUS-006</t>
         </is>
       </c>
-      <c r="E9" s="10" t="inlineStr">
-        <is>
-          <t>● Dado do TX</t>
-        </is>
-      </c>
       <c r="F9" s="45" t="inlineStr">
         <is>
-          <t>Derivado da distribuição medida no adesivo do TX/E05 (48,43 % no eixo dianteiro, com piloto) × wheelbase; coerente com a massa total, que inclui o piloto.</t>
-        </is>
-      </c>
-      <c r="G9" s="10" t="n">
-        <v>0.82203</v>
-      </c>
-      <c r="H9" s="10" t="inlineStr">
-        <is>
-          <t>● Dado do TX</t>
+          <t>Calculada (EDR-050): L·(1 − f), com f = fração de peso no eixo dianteiro (B32).</t>
         </is>
       </c>
     </row>
@@ -10218,8 +10200,9 @@
           <t>CG -&gt; eixo traseiro (b)</t>
         </is>
       </c>
-      <c r="B10" s="16" t="n">
-        <v>0.77197</v>
+      <c r="B10" s="21">
+        <f>'05_VEHICLE'!$B$6*'05_VEHICLE'!$B$32</f>
+        <v/>
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
@@ -10231,22 +10214,9 @@
           <t>SUS-006</t>
         </is>
       </c>
-      <c r="E10" s="10" t="inlineStr">
-        <is>
-          <t>● Dado do TX</t>
-        </is>
-      </c>
       <c r="F10" s="45" t="inlineStr">
         <is>
-          <t>Derivado da distribuição medida no adesivo do TX/E05 (51,57 % no eixo traseiro, com piloto) × wheelbase.</t>
-        </is>
-      </c>
-      <c r="G10" s="10" t="n">
-        <v>0.77197</v>
-      </c>
-      <c r="H10" s="10" t="inlineStr">
-        <is>
-          <t>● Dado do TX</t>
+          <t>Calculada (EDR-050): L·f, com f = fração de peso no eixo dianteiro (B32).</t>
         </is>
       </c>
     </row>
@@ -10351,8 +10321,9 @@
           <t>Altura CG não-suspenso dianteiro</t>
         </is>
       </c>
-      <c r="B16" s="16" t="n">
-        <v>0.254</v>
+      <c r="B16" s="21">
+        <f>'05_VEHICLE'!$B$33*0.0254/2</f>
+        <v/>
       </c>
       <c r="C16" s="10" t="inlineStr">
         <is>
@@ -10364,22 +10335,9 @@
           <t>SUS-010</t>
         </is>
       </c>
-      <c r="E16" s="10" t="inlineStr">
-        <is>
-          <t>○ Estimativa</t>
-        </is>
-      </c>
       <c r="F16" s="45" t="inlineStr">
         <is>
-          <t>Estimativa pelo raio do pneu 20.0-13 do E03 (diâmetro 20,0 in / 2 = 0,254 m); não é medição da equipe.</t>
-        </is>
-      </c>
-      <c r="G16" s="10" t="n">
-        <v>0.254</v>
-      </c>
-      <c r="H16" s="10" t="inlineStr">
-        <is>
-          <t>○ Estimativa</t>
+          <t>Calculada (EDR-050): diâmetro do pneu (B33) × 0,0254 / 2. Estimativa: o raio do pneu aproxima a altura do CG não suspenso; não é medição da equipe.</t>
         </is>
       </c>
     </row>
@@ -10389,8 +10347,9 @@
           <t>Altura CG não-suspenso traseiro</t>
         </is>
       </c>
-      <c r="B17" s="16" t="n">
-        <v>0.254</v>
+      <c r="B17" s="21">
+        <f>'05_VEHICLE'!$B$34*0.0254/2</f>
+        <v/>
       </c>
       <c r="C17" s="10" t="inlineStr">
         <is>
@@ -10402,22 +10361,9 @@
           <t>SUS-011</t>
         </is>
       </c>
-      <c r="E17" s="10" t="inlineStr">
-        <is>
-          <t>○ Estimativa</t>
-        </is>
-      </c>
       <c r="F17" s="45" t="inlineStr">
         <is>
-          <t>Estimativa pelo raio do pneu 20.0-13 do E03 (mesmo pneu na frente e atrás); não é medição da equipe.</t>
-        </is>
-      </c>
-      <c r="G17" s="10" t="n">
-        <v>0.254</v>
-      </c>
-      <c r="H17" s="10" t="inlineStr">
-        <is>
-          <t>○ Estimativa</t>
+          <t>Calculada (EDR-050): diâmetro do pneu (B34) × 0,0254 / 2. Estimativa: o raio do pneu aproxima a altura do CG não suspenso; não é medição da equipe.</t>
         </is>
       </c>
     </row>
@@ -10577,6 +10523,204 @@
       <c r="D27" s="10" t="inlineStr">
         <is>
           <t>SUS-009</t>
+        </is>
+      </c>
+    </row>
+    <row r="28"/>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Entradas de onde saem B4, B9/B10 e B16/B17 (EDR-050: valor que sai de conta não é digitado)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Massa medida sem piloto</t>
+        </is>
+      </c>
+      <c r="B30" s="16" t="n">
+        <v>248.5</v>
+      </c>
+      <c r="C30" s="10" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D30" s="10" t="inlineStr">
+        <is>
+          <t>SUS-001</t>
+        </is>
+      </c>
+      <c r="E30" s="10" t="inlineStr">
+        <is>
+          <t>● Dado do TX</t>
+        </is>
+      </c>
+      <c r="F30" s="45" t="inlineStr">
+        <is>
+          <t>Adesivo SAE Brasil 2026: medição real, sem piloto (248,5 kg).</t>
+        </is>
+      </c>
+      <c r="G30" s="10" t="n">
+        <v>248.5</v>
+      </c>
+      <c r="H30" s="10" t="inlineStr">
+        <is>
+          <t>● Dado do TX</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Massa do piloto</t>
+        </is>
+      </c>
+      <c r="B31" s="16" t="n">
+        <v>68</v>
+      </c>
+      <c r="C31" s="10" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D31" s="10" t="inlineStr">
+        <is>
+          <t>SUS-001</t>
+        </is>
+      </c>
+      <c r="E31" s="10" t="inlineStr">
+        <is>
+          <t>○ Estimativa</t>
+        </is>
+      </c>
+      <c r="F31" s="45" t="inlineStr">
+        <is>
+          <t>Piloto de referência (68 kg, padrão FSAE); não é a massa medida do piloto.</t>
+        </is>
+      </c>
+      <c r="G31" s="10" t="n">
+        <v>68</v>
+      </c>
+      <c r="H31" s="10" t="inlineStr">
+        <is>
+          <t>○ Estimativa</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Fração de peso no eixo dianteiro (f)</t>
+        </is>
+      </c>
+      <c r="B32" s="16" t="n">
+        <v>0.4843</v>
+      </c>
+      <c r="C32" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D32" s="10" t="inlineStr">
+        <is>
+          <t>SUS-006</t>
+        </is>
+      </c>
+      <c r="E32" s="10" t="inlineStr">
+        <is>
+          <t>● Dado do TX</t>
+        </is>
+      </c>
+      <c r="F32" s="45" t="inlineStr">
+        <is>
+          <t>Distribuição medida no adesivo do TX/E05: 48,43 % no eixo dianteiro, com piloto (coerente com a massa total, que inclui o piloto).</t>
+        </is>
+      </c>
+      <c r="G32" s="10" t="n">
+        <v>0.4843</v>
+      </c>
+      <c r="H32" s="10" t="inlineStr">
+        <is>
+          <t>● Dado do TX</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Diâmetro do pneu dianteiro</t>
+        </is>
+      </c>
+      <c r="B33" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="C33" s="10" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D33" s="10" t="inlineStr">
+        <is>
+          <t>SUS-010</t>
+        </is>
+      </c>
+      <c r="E33" s="10" t="inlineStr">
+        <is>
+          <t>◐ Dado do T09</t>
+        </is>
+      </c>
+      <c r="F33" s="45" t="inlineStr">
+        <is>
+          <t>Pneu 20.0-13 do E03 (diâmetro 20,0 in).</t>
+        </is>
+      </c>
+      <c r="G33" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="H33" s="10" t="inlineStr">
+        <is>
+          <t>◐ Dado do T09</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Diâmetro do pneu traseiro</t>
+        </is>
+      </c>
+      <c r="B34" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="C34" s="10" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D34" s="10" t="inlineStr">
+        <is>
+          <t>SUS-011</t>
+        </is>
+      </c>
+      <c r="E34" s="10" t="inlineStr">
+        <is>
+          <t>◐ Dado do T09</t>
+        </is>
+      </c>
+      <c r="F34" s="45" t="inlineStr">
+        <is>
+          <t>Pneu 20.0-13 do E03 (mesmo pneu na frente e atrás).</t>
+        </is>
+      </c>
+      <c r="G34" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="H34" s="10" t="inlineStr">
+        <is>
+          <t>◐ Dado do T09</t>
         </is>
       </c>
     </row>
@@ -10588,7 +10732,7 @@
     <mergeCell ref="A22:E22"/>
     <mergeCell ref="A3:E3"/>
   </mergeCells>
-  <conditionalFormatting sqref="E3:E27">
+  <conditionalFormatting sqref="E3:E34">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
       <formula>AND(ISNUMBER($G3),$B3&lt;&gt;$G3,$E3=$H3)</formula>
     </cfRule>
@@ -10605,13 +10749,13 @@
       <formula>LEFT($E3,1)="?"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F3:F27">
+  <conditionalFormatting sqref="F3:F34">
     <cfRule type="expression" priority="2" dxfId="5" stopIfTrue="1">
       <formula>AND(LEFT($E3,1)="●",LEN(TRIM($F3))=0)</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="E4 E5 E6 E7 E8 E9 E10 E14 E15 E16 E17 E20" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Origem fora da lista" error="Escolha uma das origens da lista (00_README, 'Como preencher')." type="list">
+    <dataValidation sqref="E5 E6 E7 E8 E14 E15 E20 E30 E31 E32 E33 E34" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Origem fora da lista" error="Escolha uma das origens da lista (00_README, 'Como preencher')." type="list">
       <formula1>=Origens</formula1>
     </dataValidation>
   </dataValidations>
@@ -13296,7 +13440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -13379,8 +13523,9 @@
           <t>Aceleração lateral (a_y)</t>
         </is>
       </c>
-      <c r="B5" s="16" t="n">
-        <v>11.772</v>
+      <c r="B5" s="21">
+        <f>'08_VEHICLE_STATE'!$B$11*9.81</f>
+        <v/>
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
@@ -13392,22 +13537,9 @@
           <t>-</t>
         </is>
       </c>
-      <c r="E5" s="10" t="inlineStr">
-        <is>
-          <t>○ Estimativa</t>
-        </is>
-      </c>
       <c r="F5" s="45" t="inlineStr">
         <is>
-          <t>Caso de carga sem fonte registrada. Curva à esquerda de 1,2 g. ISO 8855: a_y + = para a esquerda (o lado direito ganha carga).</t>
-        </is>
-      </c>
-      <c r="G5" s="10" t="n">
-        <v>11.772</v>
-      </c>
-      <c r="H5" s="10" t="inlineStr">
-        <is>
-          <t>○ Estimativa</t>
+          <t>Calculada (EDR-050): a_y em g (B11) × 9,81. ISO 8855: a_y + = para a esquerda (o lado direito ganha carga).</t>
         </is>
       </c>
     </row>
@@ -13490,6 +13622,45 @@
         <v>0.45</v>
       </c>
       <c r="H9" s="10" t="inlineStr">
+        <is>
+          <t>○ Estimativa</t>
+        </is>
+      </c>
+    </row>
+    <row r="10"/>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Aceleração lateral em g (entrada de a_y)</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>○ Estimativa</t>
+        </is>
+      </c>
+      <c r="F11" s="45" t="inlineStr">
+        <is>
+          <t>Caso de carga sem fonte registrada. Curva à esquerda de 1,2 g.</t>
+        </is>
+      </c>
+      <c r="G11" s="10" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="H11" s="10" t="inlineStr">
         <is>
           <t>○ Estimativa</t>
         </is>
@@ -13501,7 +13672,7 @@
     <mergeCell ref="A7:E7"/>
     <mergeCell ref="A3:E3"/>
   </mergeCells>
-  <conditionalFormatting sqref="E3:E9">
+  <conditionalFormatting sqref="E3:E11">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
       <formula>AND(ISNUMBER($G3),$B3&lt;&gt;$G3,$E3=$H3)</formula>
     </cfRule>
@@ -13518,13 +13689,13 @@
       <formula>LEFT($E3,1)="?"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F3:F9">
+  <conditionalFormatting sqref="F3:F11">
     <cfRule type="expression" priority="2" dxfId="5" stopIfTrue="1">
       <formula>AND(LEFT($E3,1)="●",LEN(TRIM($F3))=0)</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="E4 E5 E8 E9" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Origem fora da lista" error="Escolha uma das origens da lista (00_README, 'Como preencher')." type="list">
+    <dataValidation sqref="E4 E8 E9 E11" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Origem fora da lista" error="Escolha uma das origens da lista (00_README, 'Como preencher')." type="list">
       <formula1>=Origens</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
fix: ajustes da revisão do PR na 2ª rodada da V3.0
- Guia da 00_README avisa que a 10_TIRE não tem os avisos de origem.
- 08_VEHICLE_STATE ganha cabeçalho (A10) para a entrada de a_y em g.
- Gerador para se o texto de 00_README!A3 mudar (o replace era silencioso).
- TC-WB30-010: raízes da V2.1 que viraram fórmula (05 B16/B17, 08 B5) são
  exceção explícita, com a categoria conferida na Fonte.
- TC-WB30-011: legenda comparada com as cores esperadas, não só com a
  célula de onde o estilo foi copiado.

Suíte inteira PASS (362 fórmulas; test_workbook_suspensao 13/13).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel/FSAE_EV_Suspension_Fase1_V3_0.xlsx
+++ b/excel/FSAE_EV_Suspension_Fase1_V3_0.xlsx
@@ -1229,7 +1229,7 @@
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>3. Avisos: Origem com fundo vermelho-alaranjado = o valor mudou e a Origem continuou a mesma (revise a Origem). Fonte com fundo vermelho = a Origem diz "Dado do TX" e falta a Fonte.</t>
+          <t>3. Avisos: Origem com fundo vermelho-alaranjado = o valor mudou e a Origem continuou a mesma (revise a Origem). Fonte com fundo vermelho = a Origem diz "Dado do TX" e falta a Fonte. Na 10_TIRE não há esses avisos: ao trocar um caso de carga, troque a Origem à mão.</t>
         </is>
       </c>
     </row>
@@ -13627,7 +13627,13 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Entrada de onde sai a_y (B5) — EDR-050</t>
+        </is>
+      </c>
+    </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs: renomeia a rodada do feedback da equipe para "1ª rodada de feedback"
Numeração pedida pelo usuário (2026-10-19): a revisão metodológica abriu a
V3.0 e as rodadas de feedback contam à parte. O trabalho do PR #9, antes
chamado de "2ª rodada", é a 1ª rodada de feedback; a próxima é a 2ª.

Só texto: documentos, comentários, docstrings e os textos da 00_README!A3 e
da 15_CHANGELOG (planilha regenerada pelo atualizar_planilha.py). Nenhuma
fórmula muda (362). Suíte inteira PASS.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel/FSAE_EV_Suspension_Fase1_V3_0.xlsx
+++ b/excel/FSAE_EV_Suspension_Fase1_V3_0.xlsx
@@ -846,7 +846,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Versão do workbook: V3.0 (em desenvolvimento até concluir as correções de feedback; revisão metodológica contra Milliken/Gillespie/Seward/Pacejka: pneu em série, termo gravitacional da rolagem, massa suspensa por eixo, anti com sinal, Ky com um λFz0; EDR-045 a EDR-049; 2ª rodada, feedback da equipe: origem de cada entrada, valores derivados como fórmula, guia de preenchimento; EDR-035, EDR-050, EDR-051) | Status: DRAFT — cross-check, ainda NÃO REFERENCE-validated</t>
+          <t>Versão do workbook: V3.0 (em desenvolvimento até concluir as correções de feedback; revisão metodológica contra Milliken/Gillespie/Seward/Pacejka: pneu em série, termo gravitacional da rolagem, massa suspensa por eixo, anti com sinal, Ky com um λFz0; EDR-045 a EDR-049; 1ª rodada de feedback (da equipe): origem de cada entrada, valores derivados como fórmula, guia de preenchimento; EDR-035, EDR-050, EDR-051) | Status: DRAFT — cross-check, ainda NÃO REFERENCE-validated</t>
         </is>
       </c>
     </row>
@@ -8500,7 +8500,7 @@
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>V3.0, 2a rodada (feedback da equipe): coluna Origem (lista) e Fonte em cada entrada (05, 06, 07, 08, 11; 10_TIRE I/J), com cores e aviso de origem desatualizada; fundo amarelo retirado e legenda corrigida; valores derivados como formula (05_VEHICLE B4, B9, B10, B16, B17; 08 B5; entradas novas 05 B30:B34 e 08 B11); guia 'Como preencher' na 00_README.</t>
+          <t>V3.0, 1a rodada de feedback (da equipe): coluna Origem (lista) e Fonte em cada entrada (05, 06, 07, 08, 11; 10_TIRE I/J), com cores e aviso de origem desatualizada; fundo amarelo retirado e legenda corrigida; valores derivados como formula (05_VEHICLE B4, B9, B10, B16, B17; 08 B5; entradas novas 05 B30:B34 e 08 B11); guia 'Como preencher' na 00_README.</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">

</xml_diff>

<commit_message>
feat: hipótese do CG não suspenso vira entrada e centro da roda sai do SUS-011
2ª rodada de feedback da V3.0 (decisões do usuário em 2026-10-19).

- 05_VEHICLE B35/B36: razão h_ns / raio do pneu (1,0, Estimativa; Milliken
  p. 672). B16/B17 = raio x razão (EDR-050: parcela externa vira entrada).
- 07_KINEMATICS B14 (centro da roda traseira, anti-squat) apontava para
  05 B17, a mesma célula do CG não suspenso; passa a usar o raio direto,
  para que a razão não mova o ponto de reação.
- Item 7 do guia da 00_README: significado de N/A e TBD (EDR-035). Fica
  no mesmo commit porque a planilha é um único arquivo gerado.

Nenhum valor muda (razão 1); 362 fórmulas. TC-WB30-013 estendido e
TC-WB30-005 com a razão perturbada; suíte inteira PASS.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel/FSAE_EV_Suspension_Fase1_V3_0.xlsx
+++ b/excel/FSAE_EV_Suspension_Fase1_V3_0.xlsx
@@ -825,7 +825,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -846,7 +846,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Versão do workbook: V3.0 (em desenvolvimento até concluir as correções de feedback; revisão metodológica contra Milliken/Gillespie/Seward/Pacejka: pneu em série, termo gravitacional da rolagem, massa suspensa por eixo, anti com sinal, Ky com um λFz0; EDR-045 a EDR-049; 1ª rodada de feedback (da equipe): origem de cada entrada, valores derivados como fórmula, guia de preenchimento; EDR-035, EDR-050, EDR-051) | Status: DRAFT — cross-check, ainda NÃO REFERENCE-validated</t>
+          <t>Versão do workbook: V3.0 (em desenvolvimento até concluir as correções de feedback; revisão metodológica contra Milliken/Gillespie/Seward/Pacejka: pneu em série, termo gravitacional da rolagem, massa suspensa por eixo, anti com sinal, Ky com um λFz0; EDR-045 a EDR-049; 1ª rodada de feedback (da equipe): origem de cada entrada, valores derivados como fórmula, guia de preenchimento; EDR-035, EDR-050, EDR-051; 2ª rodada de feedback: hipótese do CG não suspenso como entrada, centro da roda separado, significado de N/A e TBD) | Status: DRAFT — cross-check, ainda NÃO REFERENCE-validated</t>
         </is>
       </c>
     </row>
@@ -1254,8 +1254,15 @@
         </is>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>7. N/A = não se aplica, ou não dá para calcular na configuração atual (falta dado, valor fora da faixa do pneu, instabilidade): a célula nunca mostra número inventado. TBD = falta um dado, uma meta ou uma decisão (equivale a OPEN). "? A confirmar" (coluna Origem) é outra coisa: há valor, mas a origem dele não está registrada.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="45">
+  <mergeCells count="46">
     <mergeCell ref="A30:E30"/>
     <mergeCell ref="A39:E39"/>
     <mergeCell ref="A34:E34"/>
@@ -1289,6 +1296,7 @@
     <mergeCell ref="A8:E8"/>
     <mergeCell ref="A22:E22"/>
     <mergeCell ref="B47:D47"/>
+    <mergeCell ref="A53:E53"/>
     <mergeCell ref="B17:E17"/>
     <mergeCell ref="A35:E35"/>
     <mergeCell ref="B46:D46"/>
@@ -8236,7 +8244,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8506,6 +8514,23 @@
       <c r="C17" s="12" t="inlineStr">
         <is>
           <t>Feedback da equipe (2026-10-14) e decisoes do usuario (2026-10-19). EDR-025 (A), EDR-035, EDR-050, EDR-051. Registro celula a celula: docs/registro-de-versoes-V3_0.md. Validation: test_workbook_suspensao (TC-WB30-010..013). NOT_VALIDATED fisicamente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>V3.0, 2a rodada de feedback: razao h_ns / raio do pneu como entrada (05_VEHICLE B35/B36, Milliken p. 672); 05 B16/B17 = raio x razao; 07_KINEMATICS B14 (centro da roda traseira) = raio do pneu, sem passar pelo CG nao suspenso; item 7 do guia (N/A e TBD).</t>
+        </is>
+      </c>
+      <c r="C18" s="12" t="inlineStr">
+        <is>
+          <t>Decisoes do usuario (2026-10-19). EDR-050 (estendido), EDR-035 (N/A e TBD). Registro celula a celula: docs/registro-de-versoes-V3_0.md. Validation: test_workbook_suspensao (TC-WB30-013 estendido). NOT_VALIDATED fisicamente.</t>
         </is>
       </c>
     </row>
@@ -9951,7 +9976,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -10322,7 +10347,7 @@
         </is>
       </c>
       <c r="B16" s="21">
-        <f>'05_VEHICLE'!$B$33*0.0254/2</f>
+        <f>'05_VEHICLE'!$B$33*0.0254/2*'05_VEHICLE'!$B$35</f>
         <v/>
       </c>
       <c r="C16" s="10" t="inlineStr">
@@ -10337,7 +10362,7 @@
       </c>
       <c r="F16" s="45" t="inlineStr">
         <is>
-          <t>Calculada (EDR-050): diâmetro do pneu (B33) × 0,0254 / 2. Estimativa: o raio do pneu aproxima a altura do CG não suspenso; não é medição da equipe.</t>
+          <t>Calculada (EDR-050): raio do pneu (B33 × 0,0254 / 2) × razão h_ns / raio (B35). Estimativa: a hipótese está na razão (B35), não é medição da equipe.</t>
         </is>
       </c>
     </row>
@@ -10348,7 +10373,7 @@
         </is>
       </c>
       <c r="B17" s="21">
-        <f>'05_VEHICLE'!$B$34*0.0254/2</f>
+        <f>'05_VEHICLE'!$B$34*0.0254/2*'05_VEHICLE'!$B$36</f>
         <v/>
       </c>
       <c r="C17" s="10" t="inlineStr">
@@ -10363,7 +10388,7 @@
       </c>
       <c r="F17" s="45" t="inlineStr">
         <is>
-          <t>Calculada (EDR-050): diâmetro do pneu (B34) × 0,0254 / 2. Estimativa: o raio do pneu aproxima a altura do CG não suspenso; não é medição da equipe.</t>
+          <t>Calculada (EDR-050): raio do pneu (B34 × 0,0254 / 2) × razão h_ns / raio (B36). Estimativa: a hipótese está na razão (B36), não é medição da equipe.</t>
         </is>
       </c>
     </row>
@@ -10721,6 +10746,82 @@
       <c r="H34" s="10" t="inlineStr">
         <is>
           <t>◐ Dado do T09</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Razão h_ns / raio do pneu dianteiro</t>
+        </is>
+      </c>
+      <c r="B35" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="C35" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D35" s="10" t="inlineStr">
+        <is>
+          <t>SUS-010</t>
+        </is>
+      </c>
+      <c r="E35" s="10" t="inlineStr">
+        <is>
+          <t>○ Estimativa</t>
+        </is>
+      </c>
+      <c r="F35" s="45" t="inlineStr">
+        <is>
+          <t>Estimativa: Milliken p. 672 (cap. 18, altura do CG suspenso) toma a altura do centro da roda como "boa primeira aproximação" da altura do CG não suspenso e usa o raio carregado (R_LF, R_LR); razão 1 = essa aproximação. Aqui o raio é o sem carga (diâmetro / 2), sem a deflexão estática do pneu. Trocar pela medição do conjunto não suspenso quando houver.</t>
+        </is>
+      </c>
+      <c r="G35" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H35" s="10" t="inlineStr">
+        <is>
+          <t>○ Estimativa</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Razão h_ns / raio do pneu traseiro</t>
+        </is>
+      </c>
+      <c r="B36" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="C36" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D36" s="10" t="inlineStr">
+        <is>
+          <t>SUS-011</t>
+        </is>
+      </c>
+      <c r="E36" s="10" t="inlineStr">
+        <is>
+          <t>○ Estimativa</t>
+        </is>
+      </c>
+      <c r="F36" s="45" t="inlineStr">
+        <is>
+          <t>Estimativa: Milliken p. 672 (cap. 18, altura do CG suspenso) toma a altura do centro da roda como "boa primeira aproximação" da altura do CG não suspenso e usa o raio carregado (R_LF, R_LR); razão 1 = essa aproximação. Aqui o raio é o sem carga (diâmetro / 2), sem a deflexão estática do pneu. Trocar pela medição do conjunto não suspenso quando houver.</t>
+        </is>
+      </c>
+      <c r="G36" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H36" s="10" t="inlineStr">
+        <is>
+          <t>○ Estimativa</t>
         </is>
       </c>
     </row>
@@ -10732,7 +10833,7 @@
     <mergeCell ref="A22:E22"/>
     <mergeCell ref="A3:E3"/>
   </mergeCells>
-  <conditionalFormatting sqref="E3:E34">
+  <conditionalFormatting sqref="E3:E36">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
       <formula>AND(ISNUMBER($G3),$B3&lt;&gt;$G3,$E3=$H3)</formula>
     </cfRule>
@@ -10749,13 +10850,13 @@
       <formula>LEFT($E3,1)="?"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F3:F34">
+  <conditionalFormatting sqref="F3:F36">
     <cfRule type="expression" priority="2" dxfId="5" stopIfTrue="1">
       <formula>AND(LEFT($E3,1)="●",LEN(TRIM($F3))=0)</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="E5 E6 E7 E8 E14 E15 E20 E30 E31 E32 E33 E34" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Origem fora da lista" error="Escolha uma das origens da lista (00_README, 'Como preencher')." type="list">
+    <dataValidation sqref="E5 E6 E7 E8 E14 E15 E20 E30 E31 E32 E33 E34 E35 E36" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Origem fora da lista" error="Escolha uma das origens da lista (00_README, 'Como preencher')." type="list">
       <formula1>=Origens</formula1>
     </dataValidation>
   </dataValidations>
@@ -12092,7 +12193,7 @@
         </is>
       </c>
       <c r="B14" s="22">
-        <f>'05_VEHICLE'!$B$17</f>
+        <f>'05_VEHICLE'!$B$34*0.0254/2</f>
         <v/>
       </c>
       <c r="C14" s="10" t="inlineStr">
@@ -12107,7 +12208,7 @@
       </c>
       <c r="F14" s="45" t="inlineStr">
         <is>
-          <t>Calculada: = SUS-011 (05_VEHICLE B17). Placeholder: substituir pela altura do centro da roda do CAD.</t>
+          <t>Calculada: raio sem carga do pneu traseiro (05_VEHICLE B34 × 0,0254 / 2), sem a deflexão estática. Placeholder: substituir pela altura do centro da roda do CAD.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: pior origem ao vivo nos resultados do 14_DASHBOARD (FB-03 fase 2)
Aprovada pelo usuário em 2026-10-19 (2ª rodada de feedback da V3.0).
Coluna E do 14_DASHBOARD em 19 resultados: =INDEX(Origens,MAX(IFERROR(
MATCH(<origem>,Origens,0),6),...)). A lista Origens é a ordem inversa da
pior origem (? A confirmar, Arbitrário, Estimativa, TTC, T09, TX), o que
o gerador confere; origem vazia conta como ? A confirmar. As células de
origem saem do grafo de fórmulas na geração.

TC-WB30-014 (ID autorizado): cobertura das raízes, valor de base e
semântica ao vivo. 362 -> 381 fórmulas; mapa V3.0 com as 19 linhas novas.
Suíte inteira PASS; test_workbook_suspensao 14/14 pelo Excel e pelo
LibreOffice.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel/FSAE_EV_Suspension_Fase1_V3_0.xlsx
+++ b/excel/FSAE_EV_Suspension_Fase1_V3_0.xlsx
@@ -7640,7 +7640,7 @@
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -7679,7 +7679,13 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
+    <row r="5">
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Coluna E: pior origem das entradas (ao vivo)</t>
+        </is>
+      </c>
+    </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
@@ -7707,6 +7713,10 @@
           <t>SUS-104</t>
         </is>
       </c>
+      <c r="E7" s="10">
+        <f>INDEX(Origens,MAX(IFERROR(MATCH('05_VEHICLE'!$E$5,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$6,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$7,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$8,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$14,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$15,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$30,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$31,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$32,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$33,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$34,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$35,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$36,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$4,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$5,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$6,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$7,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$10,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$11,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$14,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$15,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$47,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$48,Origens,0),6),IFERROR(MATCH('08_VEHICLE_STATE'!$E$4,Origens,0),6),IFERROR(MATCH('08_VEHICLE_STATE'!$E$8,Origens,0),6),IFERROR(MATCH('08_VEHICLE_STATE'!$E$9,Origens,0),6),IFERROR(MATCH('08_VEHICLE_STATE'!$E$11,Origens,0),6)))</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -7728,6 +7738,10 @@
           <t>SUS-104</t>
         </is>
       </c>
+      <c r="E8" s="10">
+        <f>INDEX(Origens,MAX(IFERROR(MATCH('05_VEHICLE'!$E$5,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$6,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$7,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$8,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$14,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$15,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$30,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$31,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$32,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$33,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$34,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$35,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$36,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$4,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$5,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$6,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$7,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$10,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$11,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$14,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$15,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$47,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$48,Origens,0),6),IFERROR(MATCH('08_VEHICLE_STATE'!$E$4,Origens,0),6),IFERROR(MATCH('08_VEHICLE_STATE'!$E$8,Origens,0),6),IFERROR(MATCH('08_VEHICLE_STATE'!$E$9,Origens,0),6),IFERROR(MATCH('08_VEHICLE_STATE'!$E$11,Origens,0),6)))</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -7749,6 +7763,10 @@
           <t>SUS-104</t>
         </is>
       </c>
+      <c r="E9" s="10">
+        <f>INDEX(Origens,MAX(IFERROR(MATCH('05_VEHICLE'!$E$5,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$6,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$7,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$8,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$14,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$15,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$30,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$31,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$32,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$33,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$34,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$35,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$36,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$4,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$5,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$6,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$7,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$10,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$11,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$14,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$15,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$47,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$48,Origens,0),6),IFERROR(MATCH('08_VEHICLE_STATE'!$E$4,Origens,0),6),IFERROR(MATCH('08_VEHICLE_STATE'!$E$8,Origens,0),6),IFERROR(MATCH('08_VEHICLE_STATE'!$E$9,Origens,0),6),IFERROR(MATCH('08_VEHICLE_STATE'!$E$11,Origens,0),6)))</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -7769,6 +7787,10 @@
         <is>
           <t>SUS-104</t>
         </is>
+      </c>
+      <c r="E10" s="10">
+        <f>INDEX(Origens,MAX(IFERROR(MATCH('05_VEHICLE'!$E$5,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$6,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$7,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$8,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$14,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$15,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$30,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$31,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$32,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$33,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$34,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$35,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$36,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$4,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$5,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$6,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$7,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$10,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$11,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$14,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$15,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$47,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$48,Origens,0),6),IFERROR(MATCH('08_VEHICLE_STATE'!$E$4,Origens,0),6),IFERROR(MATCH('08_VEHICLE_STATE'!$E$8,Origens,0),6),IFERROR(MATCH('08_VEHICLE_STATE'!$E$9,Origens,0),6),IFERROR(MATCH('08_VEHICLE_STATE'!$E$11,Origens,0),6)))</f>
+        <v/>
       </c>
     </row>
     <row r="11"/>
@@ -7799,6 +7821,10 @@
           <t>SUS-202</t>
         </is>
       </c>
+      <c r="E13" s="10">
+        <f>INDEX(Origens,MAX(IFERROR(MATCH('06_SUSPENSION'!$E$4,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$6,Origens,0),6)))</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -7820,6 +7846,10 @@
           <t>SUS-202</t>
         </is>
       </c>
+      <c r="E14" s="10">
+        <f>INDEX(Origens,MAX(IFERROR(MATCH('06_SUSPENSION'!$E$5,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$7,Origens,0),6)))</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -7841,6 +7871,10 @@
           <t>SUS-205</t>
         </is>
       </c>
+      <c r="E15" s="10">
+        <f>INDEX(Origens,MAX(IFERROR(MATCH('05_VEHICLE'!$E$6,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$14,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$30,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$31,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$32,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$4,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$6,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$47,Origens,0),6)))</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -7862,6 +7896,10 @@
           <t>SUS-205</t>
         </is>
       </c>
+      <c r="E16" s="10">
+        <f>INDEX(Origens,MAX(IFERROR(MATCH('05_VEHICLE'!$E$6,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$15,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$30,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$31,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$32,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$5,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$7,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$48,Origens,0),6)))</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -7882,6 +7920,10 @@
         <is>
           <t>SUS-208</t>
         </is>
+      </c>
+      <c r="E17" s="10">
+        <f>INDEX(Origens,MAX(IFERROR(MATCH('05_VEHICLE'!$E$7,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$8,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$4,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$5,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$6,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$7,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$10,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$11,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$47,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$48,Origens,0),6)))</f>
+        <v/>
       </c>
     </row>
     <row r="18"/>
@@ -7912,6 +7954,10 @@
           <t>-</t>
         </is>
       </c>
+      <c r="E20" s="10">
+        <f>INDEX(Origens,MAX(IFERROR(MATCH('05_VEHICLE'!$E$5,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$6,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$7,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$8,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$14,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$15,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$30,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$31,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$32,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$33,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$34,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$35,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$36,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$4,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$5,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$6,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$7,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$10,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$11,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$14,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$15,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$47,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$48,Origens,0),6),IFERROR(MATCH('08_VEHICLE_STATE'!$E$4,Origens,0),6),IFERROR(MATCH('08_VEHICLE_STATE'!$E$8,Origens,0),6),IFERROR(MATCH('08_VEHICLE_STATE'!$E$9,Origens,0),6),IFERROR(MATCH('08_VEHICLE_STATE'!$E$11,Origens,0),6)))</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -7933,6 +7979,10 @@
           <t>-</t>
         </is>
       </c>
+      <c r="E21" s="10">
+        <f>INDEX(Origens,MAX(IFERROR(MATCH('05_VEHICLE'!$E$5,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$6,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$7,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$8,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$14,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$15,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$30,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$31,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$32,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$33,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$34,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$35,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$36,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$4,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$5,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$6,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$7,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$10,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$11,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$14,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$15,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$47,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$48,Origens,0),6),IFERROR(MATCH('08_VEHICLE_STATE'!$E$11,Origens,0),6)))</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -7954,6 +8004,10 @@
           <t>-</t>
         </is>
       </c>
+      <c r="E22" s="10">
+        <f>INDEX(Origens,MAX(IFERROR(MATCH('05_VEHICLE'!$E$5,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$7,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$8,Origens,0),6)))</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -7975,6 +8029,10 @@
           <t>-</t>
         </is>
       </c>
+      <c r="E23" s="10">
+        <f>INDEX(Origens,MAX(IFERROR(MATCH('07_KINEMATICS'!$E$31,Origens,0),6)))</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -7995,6 +8053,10 @@
         <is>
           <t>-</t>
         </is>
+      </c>
+      <c r="E24" s="10">
+        <f>INDEX(Origens,MAX(IFERROR(MATCH('07_KINEMATICS'!$E$32,Origens,0),6)))</f>
+        <v/>
       </c>
     </row>
     <row r="25"/>
@@ -8117,6 +8179,10 @@
           <t>SUS-501</t>
         </is>
       </c>
+      <c r="E33" s="10">
+        <f>INDEX(Origens,MAX(IFERROR(MATCH('10_TIRE'!$I$11,Origens,0),6),IFERROR(MATCH('10_TIRE'!$I$84,Origens,0),6)))</f>
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
@@ -8138,6 +8204,10 @@
           <t>SUS-503</t>
         </is>
       </c>
+      <c r="E34" s="10">
+        <f>INDEX(Origens,MAX(IFERROR(MATCH('05_VEHICLE'!$E$5,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$6,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$7,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$8,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$14,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$15,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$30,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$31,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$32,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$33,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$34,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$35,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$36,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$4,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$5,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$6,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$7,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$10,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$11,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$14,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$15,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$47,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$48,Origens,0),6),IFERROR(MATCH('08_VEHICLE_STATE'!$E$4,Origens,0),6),IFERROR(MATCH('08_VEHICLE_STATE'!$E$8,Origens,0),6),IFERROR(MATCH('08_VEHICLE_STATE'!$E$9,Origens,0),6),IFERROR(MATCH('08_VEHICLE_STATE'!$E$11,Origens,0),6),IFERROR(MATCH('10_TIRE'!$I$11,Origens,0),6),IFERROR(MATCH('10_TIRE'!$I$21,Origens,0),6),IFERROR(MATCH('10_TIRE'!$I$23,Origens,0),6),IFERROR(MATCH('10_TIRE'!$I$24,Origens,0),6),IFERROR(MATCH('10_TIRE'!$I$25,Origens,0),6),IFERROR(MATCH('10_TIRE'!$I$84,Origens,0),6),IFERROR(MATCH('10_TIRE'!$I$176,Origens,0),6)))</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -8159,6 +8229,10 @@
           <t>SUS-503</t>
         </is>
       </c>
+      <c r="E35" s="10">
+        <f>INDEX(Origens,MAX(IFERROR(MATCH('05_VEHICLE'!$E$5,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$6,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$7,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$8,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$14,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$15,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$30,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$31,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$32,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$33,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$34,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$35,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$36,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$4,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$5,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$6,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$7,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$10,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$11,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$14,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$15,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$47,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$48,Origens,0),6),IFERROR(MATCH('08_VEHICLE_STATE'!$E$4,Origens,0),6),IFERROR(MATCH('08_VEHICLE_STATE'!$E$8,Origens,0),6),IFERROR(MATCH('08_VEHICLE_STATE'!$E$9,Origens,0),6),IFERROR(MATCH('08_VEHICLE_STATE'!$E$11,Origens,0),6),IFERROR(MATCH('10_TIRE'!$I$11,Origens,0),6),IFERROR(MATCH('10_TIRE'!$I$21,Origens,0),6),IFERROR(MATCH('10_TIRE'!$I$23,Origens,0),6),IFERROR(MATCH('10_TIRE'!$I$24,Origens,0),6),IFERROR(MATCH('10_TIRE'!$I$25,Origens,0),6),IFERROR(MATCH('10_TIRE'!$I$84,Origens,0),6),IFERROR(MATCH('10_TIRE'!$I$176,Origens,0),6)))</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
@@ -8180,6 +8254,10 @@
           <t>SUS-503</t>
         </is>
       </c>
+      <c r="E36" s="10">
+        <f>INDEX(Origens,MAX(IFERROR(MATCH('05_VEHICLE'!$E$5,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$6,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$7,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$8,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$14,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$15,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$30,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$31,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$32,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$33,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$34,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$35,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$36,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$4,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$5,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$6,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$7,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$10,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$11,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$14,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$15,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$47,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$48,Origens,0),6),IFERROR(MATCH('08_VEHICLE_STATE'!$E$4,Origens,0),6),IFERROR(MATCH('08_VEHICLE_STATE'!$E$8,Origens,0),6),IFERROR(MATCH('08_VEHICLE_STATE'!$E$9,Origens,0),6),IFERROR(MATCH('08_VEHICLE_STATE'!$E$11,Origens,0),6),IFERROR(MATCH('10_TIRE'!$I$11,Origens,0),6),IFERROR(MATCH('10_TIRE'!$I$21,Origens,0),6),IFERROR(MATCH('10_TIRE'!$I$23,Origens,0),6),IFERROR(MATCH('10_TIRE'!$I$24,Origens,0),6),IFERROR(MATCH('10_TIRE'!$I$25,Origens,0),6),IFERROR(MATCH('10_TIRE'!$I$84,Origens,0),6),IFERROR(MATCH('10_TIRE'!$I$176,Origens,0),6)))</f>
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
@@ -8200,6 +8278,10 @@
         <is>
           <t>SUS-503</t>
         </is>
+      </c>
+      <c r="E37" s="10">
+        <f>INDEX(Origens,MAX(IFERROR(MATCH('05_VEHICLE'!$E$5,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$6,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$7,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$8,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$14,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$15,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$30,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$31,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$32,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$33,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$34,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$35,Origens,0),6),IFERROR(MATCH('05_VEHICLE'!$E$36,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$4,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$5,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$6,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$7,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$10,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$11,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$14,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$15,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$47,Origens,0),6),IFERROR(MATCH('06_SUSPENSION'!$E$48,Origens,0),6),IFERROR(MATCH('08_VEHICLE_STATE'!$E$4,Origens,0),6),IFERROR(MATCH('08_VEHICLE_STATE'!$E$8,Origens,0),6),IFERROR(MATCH('08_VEHICLE_STATE'!$E$9,Origens,0),6),IFERROR(MATCH('08_VEHICLE_STATE'!$E$11,Origens,0),6),IFERROR(MATCH('10_TIRE'!$I$11,Origens,0),6),IFERROR(MATCH('10_TIRE'!$I$21,Origens,0),6),IFERROR(MATCH('10_TIRE'!$I$23,Origens,0),6),IFERROR(MATCH('10_TIRE'!$I$24,Origens,0),6),IFERROR(MATCH('10_TIRE'!$I$25,Origens,0),6),IFERROR(MATCH('10_TIRE'!$I$84,Origens,0),6),IFERROR(MATCH('10_TIRE'!$I$176,Origens,0),6)))</f>
+        <v/>
       </c>
     </row>
     <row r="38">
@@ -8234,6 +8316,20 @@
     <mergeCell ref="A6:E6"/>
     <mergeCell ref="A3:E3"/>
   </mergeCells>
+  <conditionalFormatting sqref="E7:E37">
+    <cfRule type="expression" priority="1" dxfId="1">
+      <formula>LEFT($E7,1)="●"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="2">
+      <formula>LEFT($E7,1)="◐"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="3">
+      <formula>LEFT($E7,1)="○"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="4">
+      <formula>LEFT($E7,1)="?"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8525,7 +8621,7 @@
       </c>
       <c r="B18" s="12" t="inlineStr">
         <is>
-          <t>V3.0, 2a rodada de feedback: razao h_ns / raio do pneu como entrada (05_VEHICLE B35/B36, Milliken p. 672); 05 B16/B17 = raio x razao; 07_KINEMATICS B14 (centro da roda traseira) = raio do pneu, sem passar pelo CG nao suspenso; item 7 do guia (N/A e TBD).</t>
+          <t>V3.0, 2a rodada de feedback: razao h_ns / raio do pneu como entrada (05_VEHICLE B35/B36, Milliken p. 672); 05 B16/B17 = raio x razao; 07_KINEMATICS B14 (centro da roda traseira) = raio do pneu, sem passar pelo CG nao suspenso; item 7 do guia (N/A e TBD); 14_DASHBOARD coluna E: pior origem das entradas de cada resultado, ao vivo (FB-03 fase 2).</t>
         </is>
       </c>
       <c r="C18" s="12" t="inlineStr">

</xml_diff>

<commit_message>
chore: rodada passa a se chamar "2ª rodada da revisão metodológica"
Nome definido pelo usuário em 2026-10-19 (antes "2ª rodada de feedback").
Só texto: comentários, docstrings, referências de EDR, contagens do
CLAUDE.md, versão (00_README A3) e changelog (15_CHANGELOG B18) da
planilha. Nenhuma fórmula muda; suíte inteira PASS (381 fórmulas).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel/FSAE_EV_Suspension_Fase1_V3_0.xlsx
+++ b/excel/FSAE_EV_Suspension_Fase1_V3_0.xlsx
@@ -846,7 +846,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Versão do workbook: V3.0 (em desenvolvimento até concluir as correções de feedback; revisão metodológica contra Milliken/Gillespie/Seward/Pacejka: pneu em série, termo gravitacional da rolagem, massa suspensa por eixo, anti com sinal, Ky com um λFz0; EDR-045 a EDR-049; 1ª rodada de feedback (da equipe): origem de cada entrada, valores derivados como fórmula, guia de preenchimento; EDR-035, EDR-050, EDR-051; 2ª rodada de feedback: hipótese do CG não suspenso como entrada, centro da roda separado, significado de N/A e TBD) | Status: DRAFT — cross-check, ainda NÃO REFERENCE-validated</t>
+          <t>Versão do workbook: V3.0 (em desenvolvimento até concluir as correções de feedback; revisão metodológica contra Milliken/Gillespie/Seward/Pacejka: pneu em série, termo gravitacional da rolagem, massa suspensa por eixo, anti com sinal, Ky com um λFz0; EDR-045 a EDR-049; 1ª rodada de feedback (da equipe): origem de cada entrada, valores derivados como fórmula, guia de preenchimento; EDR-035, EDR-050, EDR-051; 2ª rodada da revisão metodológica: hipótese do CG não suspenso como entrada, centro da roda separado, significado de N/A e TBD) | Status: DRAFT — cross-check, ainda NÃO REFERENCE-validated</t>
         </is>
       </c>
     </row>
@@ -8621,7 +8621,7 @@
       </c>
       <c r="B18" s="12" t="inlineStr">
         <is>
-          <t>V3.0, 2a rodada de feedback: razao h_ns / raio do pneu como entrada (05_VEHICLE B35/B36, Milliken p. 672); 05 B16/B17 = raio x razao; 07_KINEMATICS B14 (centro da roda traseira) = raio do pneu, sem passar pelo CG nao suspenso; item 7 do guia (N/A e TBD); 14_DASHBOARD coluna E: pior origem das entradas de cada resultado, ao vivo (FB-03 fase 2).</t>
+          <t>V3.0, 2a rodada da revisao metodologica: razao h_ns / raio do pneu como entrada (05_VEHICLE B35/B36, Milliken p. 672); 05 B16/B17 = raio x razao; 07_KINEMATICS B14 (centro da roda traseira) = raio do pneu, sem passar pelo CG nao suspenso; item 7 do guia (N/A e TBD); 14_DASHBOARD coluna E: pior origem das entradas de cada resultado, ao vivo (FB-03 fase 2).</t>
         </is>
       </c>
       <c r="C18" s="12" t="inlineStr">

</xml_diff>

<commit_message>
feat: bloco de direção na 07_KINEMATICS (SUS-414, SUS-415, SUS-601)
EDR-052: Ackermann exato, % Ackermann, raio externo, relação pela
cremalheira e contribuição do roll steer ao gradiente de subesterço
(07_KINEMATICS l. 71-85; 6 fórmulas novas, 381 -> 387). Entradas
placeholder com origem e fonte. A Fonte das entradas de IC (07 B10:B13)
passa a pedir a definição do IC (EDR-053).

TC-WB30-015 (Excel == kinematics_model, base, entradas trocadas e a_y=0).
Suíte inteira PASS; test_workbook_suspensao 15/15 pelo Excel e pelo
LibreOffice. Mapa de raízes regenerado.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel/FSAE_EV_Suspension_Fase1_V3_0.xlsx
+++ b/excel/FSAE_EV_Suspension_Fase1_V3_0.xlsx
@@ -8622,7 +8622,7 @@
       </c>
       <c r="B18" s="12" t="inlineStr">
         <is>
-          <t>V3.0, 2a rodada da revisao metodologica: razao h_ns / raio do pneu como entrada (05_VEHICLE B35/B36, Milliken p. 672); 05 B16/B17 = raio x razao; 07_KINEMATICS B14 (centro da roda traseira) = raio do pneu, sem passar pelo CG nao suspenso; item 7 do guia (N/A e TBD); 14_DASHBOARD coluna E: pior origem das entradas de cada resultado, ao vivo (FB-03 fase 2); 10_TIRE: eixo do .tir = ISO_TYDEX (EDR-039 reaberto, help do Adams PAC2002).</t>
+          <t>V3.0, 2a rodada da revisao metodologica: razao h_ns / raio do pneu como entrada (05_VEHICLE B35/B36, Milliken p. 672); 05 B16/B17 = raio x razao; 07_KINEMATICS B14 (centro da roda traseira) = raio do pneu, sem passar pelo CG nao suspenso; item 7 do guia (N/A e TBD); 14_DASHBOARD coluna E: pior origem das entradas de cada resultado, ao vivo (FB-03 fase 2); 10_TIRE: eixo do .tir = ISO_TYDEX (EDR-039 reaberto, help do Adams PAC2002); 07_KINEMATICS l.71-85: direcao (Ackermann, relacao pela cremalheira, roll steer; SUS-414, SUS-415, SUS-601; EDR-052).</t>
         </is>
       </c>
       <c r="C18" s="12" t="inlineStr">
@@ -12047,7 +12047,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H69"/>
+  <dimension ref="A1:H85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -12157,7 +12157,7 @@
       </c>
       <c r="F10" s="45" t="inlineStr">
         <is>
-          <t>Placeholder geométrico para testar a fórmula; não é hardpoint real. Fase 2: REFERENCE do OptimumKinematics.</t>
+          <t>Placeholder geométrico para testar a fórmula; não é hardpoint real. Fase 2: REFERENCE do OptimumKinematics. Ao preencher, diga na Fonte de que definição veio o IC: linha de força pelo trabalho virtual (Python, kinematics_model.force_lines_vw; EDR-053) ou tela do OptimumKinematics (definição a confirmar). Na geometria sintética as duas dão 38,6 % e cerca de 93 % de anti-dive.</t>
         </is>
       </c>
       <c r="G10" s="10" t="n">
@@ -12195,7 +12195,7 @@
       </c>
       <c r="F11" s="45" t="inlineStr">
         <is>
-          <t>Placeholder geométrico (07_KINEMATICS inteira é placeholder até a Fase 2); não é hardpoint real.</t>
+          <t>Placeholder geométrico (07_KINEMATICS inteira é placeholder até a Fase 2); não é hardpoint real. Ao preencher, diga na Fonte de que definição veio o IC: linha de força pelo trabalho virtual (Python, kinematics_model.force_lines_vw; EDR-053) ou tela do OptimumKinematics (definição a confirmar). Na geometria sintética as duas dão 38,6 % e cerca de 93 % de anti-dive.</t>
         </is>
       </c>
       <c r="G11" s="10" t="n">
@@ -12233,7 +12233,7 @@
       </c>
       <c r="F12" s="45" t="inlineStr">
         <is>
-          <t>Placeholder geométrico (07_KINEMATICS inteira é placeholder até a Fase 2); não é hardpoint real.</t>
+          <t>Placeholder geométrico (07_KINEMATICS inteira é placeholder até a Fase 2); não é hardpoint real. Ao preencher, diga na Fonte de que definição veio o IC: linha de força pelo trabalho virtual (Python, kinematics_model.force_lines_vw; EDR-053) ou tela do OptimumKinematics (definição a confirmar). Na geometria sintética as duas dão 38,6 % e cerca de 93 % de anti-dive.</t>
         </is>
       </c>
       <c r="G12" s="10" t="n">
@@ -12271,7 +12271,7 @@
       </c>
       <c r="F13" s="45" t="inlineStr">
         <is>
-          <t>Placeholder geométrico (07_KINEMATICS inteira é placeholder até a Fase 2); não é hardpoint real.</t>
+          <t>Placeholder geométrico (07_KINEMATICS inteira é placeholder até a Fase 2); não é hardpoint real. Ao preencher, diga na Fonte de que definição veio o IC: linha de força pelo trabalho virtual (Python, kinematics_model.force_lines_vw; EDR-053) ou tela do OptimumKinematics (definição a confirmar). Na geometria sintética as duas dão 38,6 % e cerca de 93 % de anti-dive.</t>
         </is>
       </c>
       <c r="G13" s="10" t="n">
@@ -13584,15 +13584,424 @@
         </is>
       </c>
     </row>
+    <row r="70"/>
+    <row r="71">
+      <c r="A71" s="3" t="inlineStr">
+        <is>
+          <t>Direção — Ackermann (SUS-414) — entradas PLACEHOLDER até haver a medição ou a geometria do TX</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="4" t="inlineStr">
+        <is>
+          <t>Ângulo da roda dianteira externa (δo)</t>
+        </is>
+      </c>
+      <c r="B72" s="22" t="n">
+        <v>20</v>
+      </c>
+      <c r="C72" s="10" t="inlineStr">
+        <is>
+          <t>°</t>
+        </is>
+      </c>
+      <c r="D72" s="10" t="inlineStr">
+        <is>
+          <t>SUS-414</t>
+        </is>
+      </c>
+      <c r="E72" s="10" t="inlineStr">
+        <is>
+          <t>○ Estimativa</t>
+        </is>
+      </c>
+      <c r="F72" s="45" t="inlineStr">
+        <is>
+          <t>Estimativa: carros de FSAE precisam de pouco mais de 20° de esterço na roda externa (Seward p. 162-163, Tab. 6.2). Não é o batente do TX.</t>
+        </is>
+      </c>
+      <c r="G72" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="H72" s="10" t="inlineStr">
+        <is>
+          <t>○ Estimativa</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="4" t="inlineStr">
+        <is>
+          <t>Ângulo da roda dianteira interna (δi) no mesmo esterço</t>
+        </is>
+      </c>
+      <c r="B73" s="22" t="n">
+        <v>20</v>
+      </c>
+      <c r="C73" s="10" t="inlineStr">
+        <is>
+          <t>°</t>
+        </is>
+      </c>
+      <c r="D73" s="10" t="inlineStr">
+        <is>
+          <t>SUS-414</t>
+        </is>
+      </c>
+      <c r="E73" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
+      <c r="F73" s="45" t="inlineStr">
+        <is>
+          <t>Placeholder: igual a δo (direção paralela, 0 % Ackermann) até haver a medição do TX ou a geometria (Python: kinematics_model.ackermann_from_kinematics).</t>
+        </is>
+      </c>
+      <c r="G73" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="H73" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="4" t="inlineStr">
+        <is>
+          <t>δi para Ackermann exato</t>
+        </is>
+      </c>
+      <c r="B74" s="21">
+        <f>DEGREES(ATAN(1/(1/TAN(RADIANS('07_KINEMATICS'!$B$72))-'05_VEHICLE'!$B$7/'05_VEHICLE'!$B$6)))</f>
+        <v/>
+      </c>
+      <c r="C74" s="10" t="inlineStr">
+        <is>
+          <t>°</t>
+        </is>
+      </c>
+      <c r="D74" s="10" t="inlineStr">
+        <is>
+          <t>SUS-414</t>
+        </is>
+      </c>
+      <c r="F74" s="45" t="inlineStr">
+        <is>
+          <t>Calculada: cot δo − cot δi = t/L (Gillespie eq. 8-1 e 8-2, p. 277-278), com t = 05 B7 e L = 05 B6. Reproduz a Tab. 6.2 do Seward.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="4" t="inlineStr">
+        <is>
+          <t>% Ackermann</t>
+        </is>
+      </c>
+      <c r="B75" s="21">
+        <f>('07_KINEMATICS'!$B$73-'07_KINEMATICS'!$B$72)/('07_KINEMATICS'!$B$74-'07_KINEMATICS'!$B$72)*100</f>
+        <v/>
+      </c>
+      <c r="C75" s="10" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D75" s="10" t="inlineStr">
+        <is>
+          <t>SUS-414</t>
+        </is>
+      </c>
+      <c r="F75" s="45" t="inlineStr">
+        <is>
+          <t>Calculada: 100 % = Ackermann exato; 0 % = paralelo; &lt; 0 = reverso (Milliken p. 714-716; Seward, glossário). A razão entre os dois extremos é a forma adotada pelo projeto (EDR-052).</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="4" t="inlineStr">
+        <is>
+          <t>Raio da trajetória da roda dianteira externa</t>
+        </is>
+      </c>
+      <c r="B76" s="21">
+        <f>'05_VEHICLE'!$B$6/SIN(RADIANS('07_KINEMATICS'!$B$72))</f>
+        <v/>
+      </c>
+      <c r="C76" s="10" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D76" s="10" t="inlineStr">
+        <is>
+          <t>SUS-414</t>
+        </is>
+      </c>
+      <c r="F76" s="45" t="inlineStr">
+        <is>
+          <t>Calculada: L / sin δo (Seward, Tab. 6.2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="3" t="inlineStr">
+        <is>
+          <t>Direção — relação de direção pela cremalheira (SUS-601, Milliken p. 718)</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="4" t="inlineStr">
+        <is>
+          <t>Curso da cremalheira por volta do pinhão (c-factor)</t>
+        </is>
+      </c>
+      <c r="B78" s="22" t="n">
+        <v>0.0508</v>
+      </c>
+      <c r="C78" s="10" t="inlineStr">
+        <is>
+          <t>m/volta</t>
+        </is>
+      </c>
+      <c r="D78" s="10" t="inlineStr">
+        <is>
+          <t>SUS-601</t>
+        </is>
+      </c>
+      <c r="E78" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
+      <c r="F78" s="45" t="inlineStr">
+        <is>
+          <t>Placeholder: o exemplo de "2-inch rack" do Milliken p. 718; não é a cremalheira do TX.</t>
+        </is>
+      </c>
+      <c r="G78" s="10" t="n">
+        <v>0.0508</v>
+      </c>
+      <c r="H78" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="4" t="inlineStr">
+        <is>
+          <t>Comprimento do braço de direção (pino mestre à barra)</t>
+        </is>
+      </c>
+      <c r="B79" s="22" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C79" s="10" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D79" s="10" t="inlineStr">
+        <is>
+          <t>SUS-601</t>
+        </is>
+      </c>
+      <c r="E79" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
+      <c r="F79" s="45" t="inlineStr">
+        <is>
+          <t>Placeholder: valor do caso de teste TC-KIN-109 (e = 0,10 m); não é o braço do TX.</t>
+        </is>
+      </c>
+      <c r="G79" s="10" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H79" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="inlineStr">
+        <is>
+          <t>Relação de direção estimada pela cremalheira</t>
+        </is>
+      </c>
+      <c r="B80" s="21">
+        <f>360/DEGREES(ASIN('07_KINEMATICS'!$B$78/'07_KINEMATICS'!$B$79))</f>
+        <v/>
+      </c>
+      <c r="C80" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D80" s="10" t="inlineStr">
+        <is>
+          <t>SUS-601</t>
+        </is>
+      </c>
+      <c r="F80" s="45" t="inlineStr">
+        <is>
+          <t>Calculada: SR ≈ 360 / asin(c/braço), Milliken p. 718 (o livro imprime asin(c/braço)/360, que é o inverso da razão definida na p. 716; EDR-052). Vale com a barra quase perpendicular ao braço. Compare com 06_SUSPENSION B44.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="3" t="inlineStr">
+        <is>
+          <t>Direção — roll steer e gradiente de subesterço (SUS-415, Gillespie eq. 6-57)</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="4" t="inlineStr">
+        <is>
+          <t>Roll steer dianteiro (ε_f)</t>
+        </is>
+      </c>
+      <c r="B82" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="C82" s="10" t="inlineStr">
+        <is>
+          <t>°/°</t>
+        </is>
+      </c>
+      <c r="D82" s="10" t="inlineStr">
+        <is>
+          <t>SUS-415</t>
+        </is>
+      </c>
+      <c r="E82" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
+      <c r="F82" s="45" t="inlineStr">
+        <is>
+          <t>Placeholder: sem hardpoints reais. ε &gt; 0 esterça para a direita numa rolagem para a direita (Gillespie p. 220). Python: kinematics_model.roll_steer_coefficient (na geometria sintética, −0,125 °/°).</t>
+        </is>
+      </c>
+      <c r="G82" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H82" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="4" t="inlineStr">
+        <is>
+          <t>Roll steer traseiro (ε_r)</t>
+        </is>
+      </c>
+      <c r="B83" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="C83" s="10" t="inlineStr">
+        <is>
+          <t>°/°</t>
+        </is>
+      </c>
+      <c r="D83" s="10" t="inlineStr">
+        <is>
+          <t>SUS-415</t>
+        </is>
+      </c>
+      <c r="E83" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
+      <c r="F83" s="45" t="inlineStr">
+        <is>
+          <t>Placeholder: sem hardpoints reais (ver B82).</t>
+        </is>
+      </c>
+      <c r="G83" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H83" s="10" t="inlineStr">
+        <is>
+          <t>○ Arbitrário / demonstrativo</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="4" t="inlineStr">
+        <is>
+          <t>Gradiente de rolagem ∂φ/∂a_y</t>
+        </is>
+      </c>
+      <c r="B84" s="21">
+        <f>IF(AND(ISNUMBER('09_LOADS'!$B$21),'08_VEHICLE_STATE'!$B$11&lt;&gt;0),DEGREES('09_LOADS'!$B$21)/'08_VEHICLE_STATE'!$B$11,"N/A")</f>
+        <v/>
+      </c>
+      <c r="C84" s="10" t="inlineStr">
+        <is>
+          <t>°/g</t>
+        </is>
+      </c>
+      <c r="D84" s="10" t="inlineStr">
+        <is>
+          <t>SUS-415</t>
+        </is>
+      </c>
+      <c r="F84" s="45" t="inlineStr">
+        <is>
+          <t>Calculada: φ (09_LOADS B21) / a_y em g (08 B11). O φ do modelo é linear em a_y (SUS-103), então a razão é o gradiente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="4" t="inlineStr">
+        <is>
+          <t>Contribuição do roll steer ao gradiente de subesterço</t>
+        </is>
+      </c>
+      <c r="B85" s="21">
+        <f>IF(ISNUMBER('07_KINEMATICS'!$B$84),('07_KINEMATICS'!$B$82-'07_KINEMATICS'!$B$83)*'07_KINEMATICS'!$B$84,"N/A")</f>
+        <v/>
+      </c>
+      <c r="C85" s="10" t="inlineStr">
+        <is>
+          <t>°/g</t>
+        </is>
+      </c>
+      <c r="D85" s="10" t="inlineStr">
+        <is>
+          <t>SUS-415</t>
+        </is>
+      </c>
+      <c r="F85" s="45" t="inlineStr">
+        <is>
+          <t>Calculada: K = (ε_f − ε_r)·∂φ/∂a_y (Gillespie eq. 6-57); K &gt; 0 = subesterço.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="16">
     <mergeCell ref="A30:E30"/>
+    <mergeCell ref="A77:E77"/>
     <mergeCell ref="A34:E34"/>
     <mergeCell ref="A35:E35"/>
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="A26:E26"/>
+    <mergeCell ref="A81:E81"/>
     <mergeCell ref="A16:E16"/>
     <mergeCell ref="A15:E15"/>
+    <mergeCell ref="A71:E71"/>
     <mergeCell ref="A63:E63"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A6:E6"/>
@@ -13600,7 +14009,7 @@
     <mergeCell ref="A9:E9"/>
     <mergeCell ref="A3:E3"/>
   </mergeCells>
-  <conditionalFormatting sqref="E3:E69">
+  <conditionalFormatting sqref="E3:E85">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
       <formula>AND(ISNUMBER($G3),$B3&lt;&gt;$G3,$E3=$H3)</formula>
     </cfRule>
@@ -13617,13 +14026,13 @@
       <formula>LEFT($E3,1)="?"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F3:F69">
+  <conditionalFormatting sqref="F3:F85">
     <cfRule type="expression" priority="2" dxfId="5" stopIfTrue="1">
       <formula>AND(LEFT($E3,1)="●",LEN(TRIM($F3))=0)</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="E10 E11 E12 E13 E17 E18 E19 E20 E23 E24 E27 E28 E31 E32" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Origem fora da lista" error="Escolha uma das origens da lista (00_README, 'Como preencher')." type="list">
+    <dataValidation sqref="E10 E11 E12 E13 E17 E18 E19 E20 E23 E24 E27 E28 E31 E32 E72 E73 E78 E79 E82 E83" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Origem fora da lista" error="Escolha uma das origens da lista (00_README, 'Como preencher')." type="list">
       <formula1>=Origens</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
fix: λKyγ (LKYG) nos termos de camber de SHy e SVy (Adams PAC2002 eq. 41-42)
O tire_model não lia nem aplicava o LKYG. Agora lê (obrigatório) e
aplica; a 10_TIRE ganha o LKYG em B177 e as fórmulas B57:F57 (SHy) e
B64:F64 (SVy) multiplicam o termo de camber por $B$177. Com LKYG = 1 no
.tir provisório, nenhum valor muda. Usuário, 2026-10-20: "Pode corrigir".

TC-TIRE-009b/c com o LKYG (8 fatores), TC-WB24-004b com o LKYG
perturbado, mutante "LKYG ignorado em SHy" (25/25). Contagem da
cinemática no rodar_testes: 74.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel/FSAE_EV_Suspension_Fase1_V3_0.xlsx
+++ b/excel/FSAE_EV_Suspension_Fase1_V3_0.xlsx
@@ -1900,7 +1900,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J176"/>
+  <dimension ref="A1:J177"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="66" customWidth="1" min="1" max="1"/>
@@ -3242,23 +3242,23 @@
         </is>
       </c>
       <c r="B57" s="21">
-        <f>IF(B$26&lt;&gt;"OK","N/A",($B$147+$B$148*B$40)*$B$109+$B$149*B$55)</f>
+        <f>IF(B$26&lt;&gt;"OK","N/A",($B$147+$B$148*B$40)*$B$109+$B$149*B$55*$B$177)</f>
         <v/>
       </c>
       <c r="C57" s="21">
-        <f>IF(C$26&lt;&gt;"OK","N/A",($B$147+$B$148*C$40)*$B$109+$B$149*C$55)</f>
+        <f>IF(C$26&lt;&gt;"OK","N/A",($B$147+$B$148*C$40)*$B$109+$B$149*C$55*$B$177)</f>
         <v/>
       </c>
       <c r="D57" s="21">
-        <f>IF(D$26&lt;&gt;"OK","N/A",($B$147+$B$148*D$40)*$B$109+$B$149*D$55)</f>
+        <f>IF(D$26&lt;&gt;"OK","N/A",($B$147+$B$148*D$40)*$B$109+$B$149*D$55*$B$177)</f>
         <v/>
       </c>
       <c r="E57" s="21">
-        <f>IF(E$26&lt;&gt;"OK","N/A",($B$147+$B$148*E$40)*$B$109+$B$149*E$55)</f>
+        <f>IF(E$26&lt;&gt;"OK","N/A",($B$147+$B$148*E$40)*$B$109+$B$149*E$55*$B$177)</f>
         <v/>
       </c>
       <c r="F57" s="21">
-        <f>IF(F$26&lt;&gt;"OK","N/A",($B$147+$B$148*F$40)*$B$109+$B$149*F$55)</f>
+        <f>IF(F$26&lt;&gt;"OK","N/A",($B$147+$B$148*F$40)*$B$109+$B$149*F$55*$B$177)</f>
         <v/>
       </c>
       <c r="G57" s="10" t="inlineStr">
@@ -3501,23 +3501,23 @@
         </is>
       </c>
       <c r="B64" s="21">
-        <f>IF(B$26&lt;&gt;"OK","N/A",B$22*(($B$150+$B$151*B$40)*$B$110+($B$152+$B$153*B$40)*B$55)*$B$106)</f>
+        <f>IF(B$26&lt;&gt;"OK","N/A",B$22*(($B$150+$B$151*B$40)*$B$110+($B$152+$B$153*B$40)*B$55*$B$177)*$B$106)</f>
         <v/>
       </c>
       <c r="C64" s="21">
-        <f>IF(C$26&lt;&gt;"OK","N/A",C$22*(($B$150+$B$151*C$40)*$B$110+($B$152+$B$153*C$40)*C$55)*$B$106)</f>
+        <f>IF(C$26&lt;&gt;"OK","N/A",C$22*(($B$150+$B$151*C$40)*$B$110+($B$152+$B$153*C$40)*C$55*$B$177)*$B$106)</f>
         <v/>
       </c>
       <c r="D64" s="21">
-        <f>IF(D$26&lt;&gt;"OK","N/A",D$22*(($B$150+$B$151*D$40)*$B$110+($B$152+$B$153*D$40)*D$55)*$B$106)</f>
+        <f>IF(D$26&lt;&gt;"OK","N/A",D$22*(($B$150+$B$151*D$40)*$B$110+($B$152+$B$153*D$40)*D$55*$B$177)*$B$106)</f>
         <v/>
       </c>
       <c r="E64" s="21">
-        <f>IF(E$26&lt;&gt;"OK","N/A",E$22*(($B$150+$B$151*E$40)*$B$110+($B$152+$B$153*E$40)*E$55)*$B$106)</f>
+        <f>IF(E$26&lt;&gt;"OK","N/A",E$22*(($B$150+$B$151*E$40)*$B$110+($B$152+$B$153*E$40)*E$55*$B$177)*$B$106)</f>
         <v/>
       </c>
       <c r="F64" s="21">
-        <f>IF(F$26&lt;&gt;"OK","N/A",F$22*(($B$150+$B$151*F$40)*$B$110+($B$152+$B$153*F$40)*F$55)*$B$106)</f>
+        <f>IF(F$26&lt;&gt;"OK","N/A",F$22*(($B$150+$B$151*F$40)*$B$110+($B$152+$B$153*F$40)*F$55*$B$177)*$B$106)</f>
         <v/>
       </c>
       <c r="G64" s="10" t="inlineStr">
@@ -4176,7 +4176,7 @@
       </c>
       <c r="J84" s="45" t="inlineStr">
         <is>
-          <t>Todos os coeficientes da tabela abaixo (B86:B175) foram transcritos do .tir provisório (ver os metadados acima). REFERENCE por natureza (DR-011), mas o dataset é provisório. Mudou o dataset: mudar o Tire REV (01_SETUP) e reexecutar 13_VALIDATION; os resultados antigos viram STALE.</t>
+          <t>Todos os coeficientes da tabela abaixo (B86:B175 e o LKYG em B177) foram transcritos do .tir provisório (ver os metadados acima). REFERENCE por natureza (DR-011), mas o dataset é provisório. Mudou o dataset: mudar o Tire REV (01_SETUP) e reexecutar 13_VALIDATION; os resultados antigos viram STALE.</t>
         </is>
       </c>
     </row>
@@ -6459,6 +6459,31 @@
       <c r="I176" s="2" t="inlineStr">
         <is>
           <t>Hipótese de implementação (mesmo valor em tire_model_V2_2.py); efeito desprezível frente a Cx·Dx.</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="4" t="inlineStr">
+        <is>
+          <t>LKYG</t>
+        </is>
+      </c>
+      <c r="B177" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="G177" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H177" s="10" t="inlineStr">
+        <is>
+          <t>SUS-501</t>
+        </is>
+      </c>
+      <c r="I177" s="2" t="inlineStr">
+        <is>
+          <t>Escala da rigidez de camber Kyγ0 (termos de camber de SHy e SVy)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: textos de fechamento da V3.0 na planilha (EDR-051)
Só texto: versão em 00_README!A3, item 5 do guia (o que a equipe pode e
não pode fazer na planilha viva) e linha 19 do 15_CHANGELOG. Nenhuma
fórmula muda (387, CA-07 PASS).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel/FSAE_EV_Suspension_Fase1_V3_0.xlsx
+++ b/excel/FSAE_EV_Suspension_Fase1_V3_0.xlsx
@@ -847,7 +847,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Versão do workbook: V3.0 (em desenvolvimento até concluir as correções de feedback; revisão metodológica contra Milliken/Gillespie/Seward/Pacejka: pneu em série, termo gravitacional da rolagem, massa suspensa por eixo, anti com sinal, Ky com um λFz0; EDR-045 a EDR-049; 1ª rodada de feedback (da equipe): origem de cada entrada, valores derivados como fórmula, guia de preenchimento; EDR-035, EDR-050, EDR-051; 2ª rodada da revisão metodológica: hipótese do CG não suspenso como entrada, centro da roda separado, significado de N/A e TBD) | Status: DRAFT — cross-check, ainda NÃO REFERENCE-validated</t>
+          <t>Versão do workbook: V3.0 (fechada em 2026-10-20: arquivo vivo da equipe, EDR-051; revisão metodológica contra Milliken/Gillespie/Seward/Pacejka: pneu em série, termo gravitacional da rolagem, massa suspensa por eixo, anti com sinal, Ky com um λFz0; EDR-045 a EDR-049; 1ª rodada de feedback (da equipe): origem de cada entrada, valores derivados como fórmula, guia de preenchimento; EDR-035, EDR-050, EDR-051; 2ª rodada da revisão metodológica: hipótese do CG não suspenso como entrada, centro da roda separado, significado de N/A e TBD) | Status: DRAFT — cross-check, ainda NÃO REFERENCE-validated</t>
         </is>
       </c>
     </row>
@@ -1244,7 +1244,7 @@
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>5. Até a V3.0 ser fechada, esta planilha é gerada pelo script do repositório e o que for digitado nela se perde na próxima geração (EDR-051). Depois do fechamento, ela passa a ser o arquivo da equipe.</t>
+          <t>5. Esta é a planilha da equipe (V3.0 fechada, EDR-051). Preencha só as entradas (valor, Origem e Fonte), as metas da 03_TARGETS e o setup da 01_SETUP. Não insira nem apague linhas, colunas ou abas, não troque fórmula por valor e não salve pelo LibreOffice. Mudança de fórmula ou de estrutura só pelo script do repositório, com aprovação. Resultado calculado com dado novo não é validado (NOT_VALIDATED) até alguém conferir.</t>
         </is>
       </c>
     </row>
@@ -8366,7 +8366,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8653,6 +8653,23 @@
       <c r="C18" s="12" t="inlineStr">
         <is>
           <t>Decisoes do usuario (2026-10-19). EDR-050 (estendido), EDR-035 (N/A e TBD). Registro celula a celula: docs/registro-de-versoes-V3_0.md. Validation: test_workbook_suspensao (TC-WB30-013 estendido). NOT_VALIDATED fisicamente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>V3.0 fechada (2026-10-20): a planilha vira o arquivo vivo da equipe; a referencia imutavel e o arquivo da tag v3.0. FB-04 passa para a V3.1.</t>
+        </is>
+      </c>
+      <c r="C19" s="12" t="inlineStr">
+        <is>
+          <t>EDR-051 (fechamento; tratamento do CA-07 decidido por conselho, a pedido do usuario). Verificacao: tools/rodar_testes.py (CA-07 regeneracao e viva; CA-09 sobre a referencia).</t>
         </is>
       </c>
     </row>

</xml_diff>